<commit_message>
scan: seg5 2026-06-24 21:38 CST
</commit_message>
<xml_diff>
--- a/output/full_scan/batch_seq6_2026-06-24.xlsx
+++ b/output/full_scan/batch_seq6_2026-06-24.xlsx
@@ -428,7 +428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O115"/>
+  <dimension ref="A1:O116"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -2488,21 +2488,21 @@
     </row>
     <row r="39">
       <c r="A39" s="2" t="n">
-        <v>6451</v>
+        <v>6415</v>
       </c>
       <c r="B39" s="2" t="inlineStr">
         <is>
-          <t>訊芯-KY</t>
+          <t>矽力*-KY</t>
         </is>
       </c>
       <c r="C39" s="2" t="n">
         <v/>
       </c>
       <c r="D39" s="2" t="n">
-        <v>740.8604402080564</v>
+        <v>746.4619567219785</v>
       </c>
       <c r="E39" s="2" t="n">
-        <v>631</v>
+        <v>605</v>
       </c>
       <c r="F39" s="2" t="inlineStr">
         <is>
@@ -2513,16 +2513,16 @@
         <v>0</v>
       </c>
       <c r="H39" s="2" t="n">
-        <v>58.18361397546864</v>
+        <v>56.37762620987802</v>
       </c>
       <c r="I39" s="2" t="n">
-        <v>32.82769439073996</v>
+        <v>27.6027128023645</v>
       </c>
       <c r="J39" s="2" t="n">
-        <v>1.19360059530191</v>
+        <v>0.5940843579364958</v>
       </c>
       <c r="K39" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L39" s="2" t="n">
         <v>0</v>
@@ -2531,31 +2531,31 @@
         <v>-1</v>
       </c>
       <c r="N39" s="2" t="n">
-        <v>-1.94710707391653</v>
+        <v>4.010753790242312</v>
       </c>
       <c r="O39" s="2" t="inlineStr">
         <is>
-          <t>above_ema60, ema60_gt_ema120, rsi_strong, market_above_ma60, liquidity_ok, adx_trending, stronger_than_market, obv_uptrend, above_ichimoku_cloud</t>
+          <t>above_ema60, ema60_gt_ema120, rsi_strong, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, stronger_than_market, obv_uptrend, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="n">
-        <v>6218</v>
+        <v>6451</v>
       </c>
       <c r="B40" s="2" t="inlineStr">
         <is>
-          <t>豪勉</t>
+          <t>訊芯-KY</t>
         </is>
       </c>
       <c r="C40" s="2" t="n">
         <v/>
       </c>
       <c r="D40" s="2" t="n">
-        <v>739.1667840134728</v>
+        <v>740.8604402080564</v>
       </c>
       <c r="E40" s="2" t="n">
-        <v>40</v>
+        <v>631</v>
       </c>
       <c r="F40" s="2" t="inlineStr">
         <is>
@@ -2566,13 +2566,13 @@
         <v>0</v>
       </c>
       <c r="H40" s="2" t="n">
-        <v>60.11011048128925</v>
+        <v>58.18361397546864</v>
       </c>
       <c r="I40" s="2" t="n">
-        <v>14.76700577178328</v>
+        <v>32.82769439073996</v>
       </c>
       <c r="J40" s="2" t="n">
-        <v>1.598474555184994</v>
+        <v>1.19360059530191</v>
       </c>
       <c r="K40" s="2" t="n">
         <v>1</v>
@@ -2584,31 +2584,31 @@
         <v>-1</v>
       </c>
       <c r="N40" s="2" t="n">
-        <v>0.5478471647118478</v>
+        <v>-1.94710707391653</v>
       </c>
       <c r="O40" s="2" t="inlineStr">
         <is>
-          <t>above_ema60, ema60_gt_ema120, volume_break, rsi_strong, market_above_ma60, liquidity_ok, stronger_than_market, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
+          <t>above_ema60, ema60_gt_ema120, rsi_strong, market_above_ma60, liquidity_ok, adx_trending, stronger_than_market, obv_uptrend, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="n">
-        <v>6284</v>
+        <v>6218</v>
       </c>
       <c r="B41" s="2" t="inlineStr">
         <is>
-          <t>佳邦</t>
+          <t>豪勉</t>
         </is>
       </c>
       <c r="C41" s="2" t="n">
         <v/>
       </c>
       <c r="D41" s="2" t="n">
-        <v>738.1862739067764</v>
+        <v>739.1667840134728</v>
       </c>
       <c r="E41" s="2" t="n">
-        <v>101.5</v>
+        <v>40</v>
       </c>
       <c r="F41" s="2" t="inlineStr">
         <is>
@@ -2619,16 +2619,16 @@
         <v>0</v>
       </c>
       <c r="H41" s="2" t="n">
-        <v>50.55835386270363</v>
+        <v>60.11011048128925</v>
       </c>
       <c r="I41" s="2" t="n">
-        <v>40.3576147131667</v>
+        <v>14.76700577178328</v>
       </c>
       <c r="J41" s="2" t="n">
-        <v>0.3083445747874439</v>
+        <v>1.598474555184994</v>
       </c>
       <c r="K41" s="2" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="L41" s="2" t="n">
         <v>0</v>
@@ -2637,31 +2637,31 @@
         <v>-1</v>
       </c>
       <c r="N41" s="2" t="n">
-        <v>-1.109423731030575</v>
+        <v>0.5478471647118478</v>
       </c>
       <c r="O41" s="2" t="inlineStr">
         <is>
-          <t>above_ema60, ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, foreign_buy_3d, adx_trending, stronger_than_market, mfi_strong, above_ichimoku_cloud</t>
+          <t>above_ema60, ema60_gt_ema120, volume_break, rsi_strong, market_above_ma60, liquidity_ok, stronger_than_market, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="n">
-        <v>6414</v>
+        <v>6284</v>
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>樺漢</t>
+          <t>佳邦</t>
         </is>
       </c>
       <c r="C42" s="2" t="n">
         <v/>
       </c>
       <c r="D42" s="2" t="n">
-        <v>734.3580340251622</v>
+        <v>738.1862739067764</v>
       </c>
       <c r="E42" s="2" t="n">
-        <v>371</v>
+        <v>101.5</v>
       </c>
       <c r="F42" s="2" t="inlineStr">
         <is>
@@ -2672,16 +2672,16 @@
         <v>0</v>
       </c>
       <c r="H42" s="2" t="n">
-        <v>51.39294968697686</v>
+        <v>50.55835386270363</v>
       </c>
       <c r="I42" s="2" t="n">
-        <v>24.98661009243359</v>
+        <v>40.3576147131667</v>
       </c>
       <c r="J42" s="2" t="n">
-        <v>0.4723320706957996</v>
+        <v>0.3083445747874439</v>
       </c>
       <c r="K42" s="2" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="L42" s="2" t="n">
         <v>0</v>
@@ -2690,31 +2690,31 @@
         <v>-1</v>
       </c>
       <c r="N42" s="2" t="n">
-        <v>-3.113418449785199</v>
+        <v>-1.109423731030575</v>
       </c>
       <c r="O42" s="2" t="inlineStr">
         <is>
-          <t>above_ema60, ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, foreign_buy_3d, adx_trending, stronger_than_market, above_ichimoku_cloud</t>
+          <t>above_ema60, ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, foreign_buy_3d, adx_trending, stronger_than_market, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="n">
-        <v>6190</v>
+        <v>6414</v>
       </c>
       <c r="B43" s="2" t="inlineStr">
         <is>
-          <t>萬泰科</t>
+          <t>樺漢</t>
         </is>
       </c>
       <c r="C43" s="2" t="n">
         <v/>
       </c>
       <c r="D43" s="2" t="n">
-        <v>733.4511239837041</v>
+        <v>734.3580340251622</v>
       </c>
       <c r="E43" s="2" t="n">
-        <v>83.09999999999999</v>
+        <v>371</v>
       </c>
       <c r="F43" s="2" t="inlineStr">
         <is>
@@ -2725,16 +2725,16 @@
         <v>0</v>
       </c>
       <c r="H43" s="2" t="n">
-        <v>55.97087412941894</v>
+        <v>51.39294968697686</v>
       </c>
       <c r="I43" s="2" t="n">
-        <v>24.73445747218834</v>
+        <v>24.98661009243359</v>
       </c>
       <c r="J43" s="2" t="n">
-        <v>0.4155008480032824</v>
+        <v>0.4723320706957996</v>
       </c>
       <c r="K43" s="2" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="L43" s="2" t="n">
         <v>0</v>
@@ -2743,31 +2743,31 @@
         <v>-1</v>
       </c>
       <c r="N43" s="2" t="n">
-        <v>-0.2261088679734917</v>
+        <v>-3.113418449785199</v>
       </c>
       <c r="O43" s="2" t="inlineStr">
         <is>
-          <t>above_ema60, ema60_gt_ema120, rsi_strong, market_above_ma60, liquidity_ok, adx_trending, stronger_than_market, kd_golden_cross, above_ichimoku_cloud</t>
+          <t>above_ema60, ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, foreign_buy_3d, adx_trending, stronger_than_market, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="n">
-        <v>6189</v>
+        <v>6190</v>
       </c>
       <c r="B44" s="2" t="inlineStr">
         <is>
-          <t>豐藝</t>
+          <t>萬泰科</t>
         </is>
       </c>
       <c r="C44" s="2" t="n">
         <v/>
       </c>
       <c r="D44" s="2" t="n">
-        <v>726.2204100408087</v>
+        <v>733.4511239837041</v>
       </c>
       <c r="E44" s="2" t="n">
-        <v>53.4</v>
+        <v>83.09999999999999</v>
       </c>
       <c r="F44" s="2" t="inlineStr">
         <is>
@@ -2778,13 +2778,13 @@
         <v>0</v>
       </c>
       <c r="H44" s="2" t="n">
-        <v>52.34936153593862</v>
+        <v>55.97087412941894</v>
       </c>
       <c r="I44" s="2" t="n">
-        <v>27.46962124642394</v>
+        <v>24.73445747218834</v>
       </c>
       <c r="J44" s="2" t="n">
-        <v>0.5438111512347565</v>
+        <v>0.4155008480032824</v>
       </c>
       <c r="K44" s="2" t="n">
         <v>1</v>
@@ -2796,31 +2796,31 @@
         <v>-1</v>
       </c>
       <c r="N44" s="2" t="n">
-        <v>-0.214852844879362</v>
+        <v>-0.2261088679734917</v>
       </c>
       <c r="O44" s="2" t="inlineStr">
         <is>
-          <t>above_ema60, ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, obv_uptrend, dealer_buy_3d, mfi_strong, above_ichimoku_cloud</t>
+          <t>above_ema60, ema60_gt_ema120, rsi_strong, market_above_ma60, liquidity_ok, adx_trending, stronger_than_market, kd_golden_cross, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="n">
-        <v>6269</v>
+        <v>6189</v>
       </c>
       <c r="B45" s="2" t="inlineStr">
         <is>
-          <t>台郡</t>
+          <t>豐藝</t>
         </is>
       </c>
       <c r="C45" s="2" t="n">
         <v/>
       </c>
       <c r="D45" s="2" t="n">
-        <v>722.9349269338519</v>
+        <v>726.2204100408087</v>
       </c>
       <c r="E45" s="2" t="n">
-        <v>79</v>
+        <v>53.4</v>
       </c>
       <c r="F45" s="2" t="inlineStr">
         <is>
@@ -2831,16 +2831,16 @@
         <v>0</v>
       </c>
       <c r="H45" s="2" t="n">
-        <v>58.58107516899551</v>
+        <v>52.34936153593862</v>
       </c>
       <c r="I45" s="2" t="n">
-        <v>32.33493809041109</v>
+        <v>27.46962124642394</v>
       </c>
       <c r="J45" s="2" t="n">
-        <v>1.07438726486</v>
+        <v>0.5438111512347565</v>
       </c>
       <c r="K45" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L45" s="2" t="n">
         <v>0</v>
@@ -2849,31 +2849,31 @@
         <v>-1</v>
       </c>
       <c r="N45" s="2" t="n">
-        <v>1.187270914660371</v>
+        <v>-0.214852844879362</v>
       </c>
       <c r="O45" s="2" t="inlineStr">
         <is>
-          <t>above_ema60, ema60_gt_ema120, rsi_strong, market_above_ma60, liquidity_ok, adx_trending, stronger_than_market, mfi_strong, above_ichimoku_cloud</t>
+          <t>above_ema60, ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, obv_uptrend, dealer_buy_3d, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="n">
-        <v>6229</v>
+        <v>6269</v>
       </c>
       <c r="B46" s="2" t="inlineStr">
         <is>
-          <t>研通</t>
+          <t>台郡</t>
         </is>
       </c>
       <c r="C46" s="2" t="n">
         <v/>
       </c>
       <c r="D46" s="2" t="n">
-        <v>718.1465735284194</v>
+        <v>722.9349269338519</v>
       </c>
       <c r="E46" s="2" t="n">
-        <v>28.3</v>
+        <v>79</v>
       </c>
       <c r="F46" s="2" t="inlineStr">
         <is>
@@ -2884,13 +2884,13 @@
         <v>0</v>
       </c>
       <c r="H46" s="2" t="n">
-        <v>59.59110144211292</v>
+        <v>58.58107516899551</v>
       </c>
       <c r="I46" s="2" t="n">
-        <v>14.45968324206507</v>
+        <v>32.33493809041109</v>
       </c>
       <c r="J46" s="2" t="n">
-        <v>0.9439546546995602</v>
+        <v>1.07438726486</v>
       </c>
       <c r="K46" s="2" t="n">
         <v>0</v>
@@ -2902,31 +2902,31 @@
         <v>-1</v>
       </c>
       <c r="N46" s="2" t="n">
-        <v>0.1593120665500457</v>
+        <v>1.187270914660371</v>
       </c>
       <c r="O46" s="2" t="inlineStr">
         <is>
-          <t>above_ema60, ema60_gt_ema120, rsi_strong, breakout_20d, market_above_ma60, stronger_than_market, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
+          <t>above_ema60, ema60_gt_ema120, rsi_strong, market_above_ma60, liquidity_ok, adx_trending, stronger_than_market, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="n">
-        <v>6224</v>
+        <v>6229</v>
       </c>
       <c r="B47" s="2" t="inlineStr">
         <is>
-          <t>聚鼎</t>
+          <t>研通</t>
         </is>
       </c>
       <c r="C47" s="2" t="n">
         <v/>
       </c>
       <c r="D47" s="2" t="n">
-        <v>712.5988205756556</v>
+        <v>718.1465735284194</v>
       </c>
       <c r="E47" s="2" t="n">
-        <v>80.09999999999999</v>
+        <v>28.3</v>
       </c>
       <c r="F47" s="2" t="inlineStr">
         <is>
@@ -2937,16 +2937,16 @@
         <v>0</v>
       </c>
       <c r="H47" s="2" t="n">
-        <v>51.23028907297992</v>
+        <v>59.59110144211292</v>
       </c>
       <c r="I47" s="2" t="n">
-        <v>23.90159516771704</v>
+        <v>14.45968324206507</v>
       </c>
       <c r="J47" s="2" t="n">
-        <v>0.4446754661069359</v>
+        <v>0.9439546546995602</v>
       </c>
       <c r="K47" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L47" s="2" t="n">
         <v>0</v>
@@ -2955,31 +2955,31 @@
         <v>-1</v>
       </c>
       <c r="N47" s="2" t="n">
-        <v>-0.701622510040478</v>
+        <v>0.1593120665500457</v>
       </c>
       <c r="O47" s="2" t="inlineStr">
         <is>
-          <t>above_ema60, ema60_gt_ema120, market_above_ma60, liquidity_ok, adx_trending, stronger_than_market, kd_golden_cross, mfi_strong, above_ichimoku_cloud</t>
+          <t>above_ema60, ema60_gt_ema120, rsi_strong, breakout_20d, market_above_ma60, stronger_than_market, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="n">
-        <v>6222</v>
+        <v>6224</v>
       </c>
       <c r="B48" s="2" t="inlineStr">
         <is>
-          <t>立軒</t>
+          <t>聚鼎</t>
         </is>
       </c>
       <c r="C48" s="2" t="n">
         <v/>
       </c>
       <c r="D48" s="2" t="n">
-        <v>711.4602343591471</v>
+        <v>712.5988205756556</v>
       </c>
       <c r="E48" s="2" t="n">
-        <v>21.2</v>
+        <v>80.09999999999999</v>
       </c>
       <c r="F48" s="2" t="inlineStr">
         <is>
@@ -2990,13 +2990,13 @@
         <v>0</v>
       </c>
       <c r="H48" s="2" t="n">
-        <v>56.99977912296026</v>
+        <v>51.23028907297992</v>
       </c>
       <c r="I48" s="2" t="n">
-        <v>25.90585183854744</v>
+        <v>23.90159516771704</v>
       </c>
       <c r="J48" s="2" t="n">
-        <v>1.476933347387653</v>
+        <v>0.4446754661069359</v>
       </c>
       <c r="K48" s="2" t="n">
         <v>1</v>
@@ -3008,31 +3008,31 @@
         <v>-1</v>
       </c>
       <c r="N48" s="2" t="n">
-        <v>0.08281662205978201</v>
+        <v>-0.701622510040478</v>
       </c>
       <c r="O48" s="2" t="inlineStr">
         <is>
-          <t>above_ema60, ema60_gt_ema120, rsi_strong, breakout_20d, market_above_ma60, avoid_chase, adx_trending, stronger_than_market, obv_uptrend, bb_squeeze_breakout</t>
+          <t>above_ema60, ema60_gt_ema120, market_above_ma60, liquidity_ok, adx_trending, stronger_than_market, kd_golden_cross, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="n">
-        <v>6228</v>
+        <v>6222</v>
       </c>
       <c r="B49" s="2" t="inlineStr">
         <is>
-          <t>全譜</t>
+          <t>立軒</t>
         </is>
       </c>
       <c r="C49" s="2" t="n">
         <v/>
       </c>
       <c r="D49" s="2" t="n">
-        <v>699</v>
+        <v>711.4602343591471</v>
       </c>
       <c r="E49" s="2" t="n">
-        <v>21.35</v>
+        <v>21.2</v>
       </c>
       <c r="F49" s="2" t="inlineStr">
         <is>
@@ -3043,13 +3043,13 @@
         <v>0</v>
       </c>
       <c r="H49" s="2" t="n">
-        <v>51.24711783904844</v>
+        <v>56.99977912296026</v>
       </c>
       <c r="I49" s="2" t="n">
-        <v>4.107828444070493</v>
+        <v>25.90585183854744</v>
       </c>
       <c r="J49" s="2" t="n">
-        <v>6.477489330671947</v>
+        <v>1.476933347387653</v>
       </c>
       <c r="K49" s="2" t="n">
         <v>1</v>
@@ -3061,31 +3061,31 @@
         <v>-1</v>
       </c>
       <c r="N49" s="2" t="n">
-        <v>-0.0402401254162598</v>
+        <v>0.08281662205978201</v>
       </c>
       <c r="O49" s="2" t="inlineStr">
         <is>
-          <t>volume_break, market_above_ma60, avoid_chase, stronger_than_market, obv_uptrend, williams_r_recovery, mfi_strong, above_ichimoku_cloud</t>
+          <t>above_ema60, ema60_gt_ema120, rsi_strong, breakout_20d, market_above_ma60, avoid_chase, adx_trending, stronger_than_market, obv_uptrend, bb_squeeze_breakout</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="n">
-        <v>6292</v>
+        <v>6228</v>
       </c>
       <c r="B50" s="2" t="inlineStr">
         <is>
-          <t>迅德</t>
+          <t>全譜</t>
         </is>
       </c>
       <c r="C50" s="2" t="n">
         <v/>
       </c>
       <c r="D50" s="2" t="n">
-        <v>670.7844022331585</v>
+        <v>699</v>
       </c>
       <c r="E50" s="2" t="n">
-        <v>61.7</v>
+        <v>21.35</v>
       </c>
       <c r="F50" s="2" t="inlineStr">
         <is>
@@ -3096,13 +3096,13 @@
         <v>0</v>
       </c>
       <c r="H50" s="2" t="n">
-        <v>51.81667236935938</v>
+        <v>51.24711783904844</v>
       </c>
       <c r="I50" s="2" t="n">
-        <v>33.21860888331927</v>
+        <v>4.107828444070493</v>
       </c>
       <c r="J50" s="2" t="n">
-        <v>0.3365326954540341</v>
+        <v>6.477489330671947</v>
       </c>
       <c r="K50" s="2" t="n">
         <v>1</v>
@@ -3114,31 +3114,31 @@
         <v>-1</v>
       </c>
       <c r="N50" s="2" t="n">
-        <v>-0.3318728403843196</v>
+        <v>-0.0402401254162598</v>
       </c>
       <c r="O50" s="2" t="inlineStr">
         <is>
-          <t>above_ema60, ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
+          <t>volume_break, market_above_ma60, avoid_chase, stronger_than_market, obv_uptrend, williams_r_recovery, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="n">
-        <v>6237</v>
+        <v>6292</v>
       </c>
       <c r="B51" s="2" t="inlineStr">
         <is>
-          <t>驊訊</t>
+          <t>迅德</t>
         </is>
       </c>
       <c r="C51" s="2" t="n">
         <v/>
       </c>
       <c r="D51" s="2" t="n">
-        <v>661.9084176029403</v>
+        <v>670.7844022331585</v>
       </c>
       <c r="E51" s="2" t="n">
-        <v>48.3</v>
+        <v>61.7</v>
       </c>
       <c r="F51" s="2" t="inlineStr">
         <is>
@@ -3149,13 +3149,13 @@
         <v>0</v>
       </c>
       <c r="H51" s="2" t="n">
-        <v>53.68263188523778</v>
+        <v>51.81667236935938</v>
       </c>
       <c r="I51" s="2" t="n">
-        <v>21.18988940502058</v>
+        <v>33.21860888331927</v>
       </c>
       <c r="J51" s="2" t="n">
-        <v>0.6495987158208216</v>
+        <v>0.3365326954540341</v>
       </c>
       <c r="K51" s="2" t="n">
         <v>1</v>
@@ -3167,31 +3167,31 @@
         <v>-1</v>
       </c>
       <c r="N51" s="2" t="n">
-        <v>-0.258975281765599</v>
+        <v>-0.3318728403843196</v>
       </c>
       <c r="O51" s="2" t="inlineStr">
         <is>
-          <t>above_ema60, ema60_gt_ema120, market_above_ma60, liquidity_ok, adx_trending, stronger_than_market, obv_uptrend, above_ichimoku_cloud</t>
+          <t>above_ema60, ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="n">
-        <v>6265</v>
+        <v>6237</v>
       </c>
       <c r="B52" s="2" t="inlineStr">
         <is>
-          <t>方土昶</t>
+          <t>驊訊</t>
         </is>
       </c>
       <c r="C52" s="2" t="n">
         <v/>
       </c>
       <c r="D52" s="2" t="n">
-        <v>661.8860000938339</v>
+        <v>661.9084176029403</v>
       </c>
       <c r="E52" s="2" t="n">
-        <v>55.9</v>
+        <v>48.3</v>
       </c>
       <c r="F52" s="2" t="inlineStr">
         <is>
@@ -3202,16 +3202,16 @@
         <v>0</v>
       </c>
       <c r="H52" s="2" t="n">
-        <v>52.94206555133792</v>
+        <v>53.68263188523778</v>
       </c>
       <c r="I52" s="2" t="n">
-        <v>32.8392007322615</v>
+        <v>21.18988940502058</v>
       </c>
       <c r="J52" s="2" t="n">
-        <v>0.32567412581067</v>
+        <v>0.6495987158208216</v>
       </c>
       <c r="K52" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L52" s="2" t="n">
         <v>0</v>
@@ -3220,31 +3220,31 @@
         <v>-1</v>
       </c>
       <c r="N52" s="2" t="n">
-        <v>-0.6369820272284437</v>
+        <v>-0.258975281765599</v>
       </c>
       <c r="O52" s="2" t="inlineStr">
         <is>
-          <t>above_ema60, ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
+          <t>above_ema60, ema60_gt_ema120, market_above_ma60, liquidity_ok, adx_trending, stronger_than_market, obv_uptrend, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="n">
-        <v>6217</v>
+        <v>6265</v>
       </c>
       <c r="B53" s="2" t="inlineStr">
         <is>
-          <t>中探針</t>
+          <t>方土昶</t>
         </is>
       </c>
       <c r="C53" s="2" t="n">
         <v/>
       </c>
       <c r="D53" s="2" t="n">
-        <v>656.4133795074401</v>
+        <v>661.8860000938339</v>
       </c>
       <c r="E53" s="2" t="n">
-        <v>257</v>
+        <v>55.9</v>
       </c>
       <c r="F53" s="2" t="inlineStr">
         <is>
@@ -3255,13 +3255,13 @@
         <v>0</v>
       </c>
       <c r="H53" s="2" t="n">
-        <v>49.48154870348526</v>
+        <v>52.94206555133792</v>
       </c>
       <c r="I53" s="2" t="n">
-        <v>14.99084458192976</v>
+        <v>32.8392007322615</v>
       </c>
       <c r="J53" s="2" t="n">
-        <v>1.504008645422577</v>
+        <v>0.32567412581067</v>
       </c>
       <c r="K53" s="2" t="n">
         <v>0</v>
@@ -3273,31 +3273,31 @@
         <v>-1</v>
       </c>
       <c r="N53" s="2" t="n">
-        <v>1.17320702723821</v>
+        <v>-0.6369820272284437</v>
       </c>
       <c r="O53" s="2" t="inlineStr">
         <is>
-          <t>above_ema60, ema60_gt_ema120, volume_break, market_above_ma60, liquidity_ok, stronger_than_market, obv_uptrend, mfi_strong</t>
+          <t>above_ema60, ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="n">
-        <v>6196</v>
+        <v>6217</v>
       </c>
       <c r="B54" s="2" t="inlineStr">
         <is>
-          <t>帆宣</t>
+          <t>中探針</t>
         </is>
       </c>
       <c r="C54" s="2" t="n">
         <v/>
       </c>
       <c r="D54" s="2" t="n">
-        <v>654.5908204664277</v>
+        <v>656.4133795074401</v>
       </c>
       <c r="E54" s="2" t="n">
-        <v>540</v>
+        <v>257</v>
       </c>
       <c r="F54" s="2" t="inlineStr">
         <is>
@@ -3308,13 +3308,13 @@
         <v>0</v>
       </c>
       <c r="H54" s="2" t="n">
-        <v>59.80542196642869</v>
+        <v>49.48154870348526</v>
       </c>
       <c r="I54" s="2" t="n">
-        <v>38.7736723388616</v>
+        <v>14.99084458192976</v>
       </c>
       <c r="J54" s="2" t="n">
-        <v>0.4625564140753084</v>
+        <v>1.504008645422577</v>
       </c>
       <c r="K54" s="2" t="n">
         <v>0</v>
@@ -3326,31 +3326,31 @@
         <v>-1</v>
       </c>
       <c r="N54" s="2" t="n">
-        <v>-2.33821850270381</v>
+        <v>1.17320702723821</v>
       </c>
       <c r="O54" s="2" t="inlineStr">
         <is>
-          <t>above_ema60, ema60_gt_ema120, rsi_strong, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, mfi_strong, above_ichimoku_cloud</t>
+          <t>above_ema60, ema60_gt_ema120, volume_break, market_above_ma60, liquidity_ok, stronger_than_market, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="n">
-        <v>6239</v>
+        <v>6196</v>
       </c>
       <c r="B55" s="2" t="inlineStr">
         <is>
-          <t>力成</t>
+          <t>帆宣</t>
         </is>
       </c>
       <c r="C55" s="2" t="n">
         <v/>
       </c>
       <c r="D55" s="2" t="n">
-        <v>646.9632683064382</v>
+        <v>654.5908204664277</v>
       </c>
       <c r="E55" s="2" t="n">
-        <v>338</v>
+        <v>540</v>
       </c>
       <c r="F55" s="2" t="inlineStr">
         <is>
@@ -3361,16 +3361,16 @@
         <v>0</v>
       </c>
       <c r="H55" s="2" t="n">
-        <v>54.76260062399805</v>
+        <v>59.80542196642869</v>
       </c>
       <c r="I55" s="2" t="n">
-        <v>31.25447317066523</v>
+        <v>38.7736723388616</v>
       </c>
       <c r="J55" s="2" t="n">
-        <v>0.6278960959383592</v>
+        <v>0.4625564140753084</v>
       </c>
       <c r="K55" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L55" s="2" t="n">
         <v>0</v>
@@ -3379,31 +3379,31 @@
         <v>-1</v>
       </c>
       <c r="N55" s="2" t="n">
-        <v>-3.063592380689997</v>
+        <v>-2.33821850270381</v>
       </c>
       <c r="O55" s="2" t="inlineStr">
         <is>
-          <t>above_ema60, ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
+          <t>above_ema60, ema60_gt_ema120, rsi_strong, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="n">
-        <v>6423</v>
+        <v>6239</v>
       </c>
       <c r="B56" s="2" t="inlineStr">
         <is>
-          <t>億而得-創</t>
+          <t>力成</t>
         </is>
       </c>
       <c r="C56" s="2" t="n">
         <v/>
       </c>
       <c r="D56" s="2" t="n">
-        <v>639.6133137157002</v>
+        <v>646.9632683064382</v>
       </c>
       <c r="E56" s="2" t="n">
-        <v>83.2</v>
+        <v>338</v>
       </c>
       <c r="F56" s="2" t="inlineStr">
         <is>
@@ -3414,16 +3414,16 @@
         <v>0</v>
       </c>
       <c r="H56" s="2" t="n">
-        <v>39.41259265913738</v>
+        <v>54.76260062399805</v>
       </c>
       <c r="I56" s="2" t="n">
-        <v>27.02783528311505</v>
+        <v>31.25447317066523</v>
       </c>
       <c r="J56" s="2" t="n">
-        <v>0.5931108389658453</v>
+        <v>0.6278960959383592</v>
       </c>
       <c r="K56" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L56" s="2" t="n">
         <v>0</v>
@@ -3432,31 +3432,31 @@
         <v>-1</v>
       </c>
       <c r="N56" s="2" t="n">
-        <v>0.1984505419537896</v>
+        <v>-3.063592380689997</v>
       </c>
       <c r="O56" s="2" t="inlineStr">
         <is>
-          <t>macd_golden_cross, ema60_gt_ema120, market_above_ma60, avoid_chase, hist_turn_positive, adx_trending, stronger_than_market, kd_golden_cross</t>
+          <t>above_ema60, ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="2" t="n">
-        <v>6174</v>
+        <v>6423</v>
       </c>
       <c r="B57" s="2" t="inlineStr">
         <is>
-          <t>安碁</t>
+          <t>億而得-創</t>
         </is>
       </c>
       <c r="C57" s="2" t="n">
         <v/>
       </c>
       <c r="D57" s="2" t="n">
-        <v>633.1491989311398</v>
+        <v>639.6133137157002</v>
       </c>
       <c r="E57" s="2" t="n">
-        <v>50.2</v>
+        <v>83.2</v>
       </c>
       <c r="F57" s="2" t="inlineStr">
         <is>
@@ -3467,13 +3467,13 @@
         <v>0</v>
       </c>
       <c r="H57" s="2" t="n">
-        <v>57.26021349105925</v>
+        <v>39.41259265913738</v>
       </c>
       <c r="I57" s="2" t="n">
-        <v>35.91032754753927</v>
+        <v>27.02783528311505</v>
       </c>
       <c r="J57" s="2" t="n">
-        <v>0.4475546394302982</v>
+        <v>0.5931108389658453</v>
       </c>
       <c r="K57" s="2" t="n">
         <v>0</v>
@@ -3485,31 +3485,31 @@
         <v>-1</v>
       </c>
       <c r="N57" s="2" t="n">
-        <v>-0.4420677523747516</v>
+        <v>0.1984505419537896</v>
       </c>
       <c r="O57" s="2" t="inlineStr">
         <is>
-          <t>above_ema60, ema60_gt_ema120, rsi_strong, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, mfi_strong, above_ichimoku_cloud</t>
+          <t>macd_golden_cross, ema60_gt_ema120, market_above_ma60, avoid_chase, hist_turn_positive, adx_trending, stronger_than_market, kd_golden_cross</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="n">
-        <v>6449</v>
+        <v>6174</v>
       </c>
       <c r="B58" s="2" t="inlineStr">
         <is>
-          <t>鈺邦</t>
+          <t>安碁</t>
         </is>
       </c>
       <c r="C58" s="2" t="n">
         <v/>
       </c>
       <c r="D58" s="2" t="n">
-        <v>630.7874110232123</v>
+        <v>633.1491989311398</v>
       </c>
       <c r="E58" s="2" t="n">
-        <v>376</v>
+        <v>50.2</v>
       </c>
       <c r="F58" s="2" t="inlineStr">
         <is>
@@ -3520,16 +3520,16 @@
         <v>0</v>
       </c>
       <c r="H58" s="2" t="n">
-        <v>52.76122819624719</v>
+        <v>57.26021349105925</v>
       </c>
       <c r="I58" s="2" t="n">
-        <v>38.25758094489873</v>
+        <v>35.91032754753927</v>
       </c>
       <c r="J58" s="2" t="n">
-        <v>1.280051230516212</v>
+        <v>0.4475546394302982</v>
       </c>
       <c r="K58" s="2" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="L58" s="2" t="n">
         <v>0</v>
@@ -3538,31 +3538,31 @@
         <v>-1</v>
       </c>
       <c r="N58" s="2" t="n">
-        <v>-8.000260229859833</v>
+        <v>-0.4420677523747516</v>
       </c>
       <c r="O58" s="2" t="inlineStr">
         <is>
-          <t>above_ema60, ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, foreign_buy_3d, adx_trending, above_ichimoku_cloud</t>
+          <t>above_ema60, ema60_gt_ema120, rsi_strong, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="2" t="n">
-        <v>6167</v>
+        <v>6449</v>
       </c>
       <c r="B59" s="2" t="inlineStr">
         <is>
-          <t>久正</t>
+          <t>鈺邦</t>
         </is>
       </c>
       <c r="C59" s="2" t="n">
         <v/>
       </c>
       <c r="D59" s="2" t="n">
-        <v>625.0296067623552</v>
+        <v>630.7874110232123</v>
       </c>
       <c r="E59" s="2" t="n">
-        <v>12.4</v>
+        <v>376</v>
       </c>
       <c r="F59" s="2" t="inlineStr">
         <is>
@@ -3573,16 +3573,16 @@
         <v>0</v>
       </c>
       <c r="H59" s="2" t="n">
-        <v>56.37741973146306</v>
+        <v>52.76122819624719</v>
       </c>
       <c r="I59" s="2" t="n">
-        <v>12.11459489913673</v>
+        <v>38.25758094489873</v>
       </c>
       <c r="J59" s="2" t="n">
-        <v>1.562765305723996</v>
+        <v>1.280051230516212</v>
       </c>
       <c r="K59" s="2" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="L59" s="2" t="n">
         <v>0</v>
@@ -3591,31 +3591,31 @@
         <v>-1</v>
       </c>
       <c r="N59" s="2" t="n">
-        <v>0.09067385324756901</v>
+        <v>-8.000260229859833</v>
       </c>
       <c r="O59" s="2" t="inlineStr">
         <is>
-          <t>above_ema60, volume_break, rsi_strong, market_above_ma60, stronger_than_market, obv_uptrend, cci_momentum, mfi_strong</t>
+          <t>above_ema60, ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, foreign_buy_3d, adx_trending, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="n">
-        <v>6279</v>
+        <v>6167</v>
       </c>
       <c r="B60" s="2" t="inlineStr">
         <is>
-          <t>胡連</t>
+          <t>久正</t>
         </is>
       </c>
       <c r="C60" s="2" t="n">
         <v/>
       </c>
       <c r="D60" s="2" t="n">
-        <v>624.1513423914423</v>
+        <v>625.0296067623552</v>
       </c>
       <c r="E60" s="2" t="n">
-        <v>120</v>
+        <v>12.4</v>
       </c>
       <c r="F60" s="2" t="inlineStr">
         <is>
@@ -3626,13 +3626,13 @@
         <v>0</v>
       </c>
       <c r="H60" s="2" t="n">
-        <v>52.52891393379767</v>
+        <v>56.37741973146306</v>
       </c>
       <c r="I60" s="2" t="n">
-        <v>18.79887470791074</v>
+        <v>12.11459489913673</v>
       </c>
       <c r="J60" s="2" t="n">
-        <v>0.3956414609622081</v>
+        <v>1.562765305723996</v>
       </c>
       <c r="K60" s="2" t="n">
         <v>0</v>
@@ -3644,31 +3644,31 @@
         <v>-1</v>
       </c>
       <c r="N60" s="2" t="n">
-        <v>-0.2960388297891239</v>
+        <v>0.09067385324756901</v>
       </c>
       <c r="O60" s="2" t="inlineStr">
         <is>
-          <t>above_ema60, market_above_ma60, avoid_chase, liquidity_ok, stronger_than_market, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
+          <t>above_ema60, volume_break, rsi_strong, market_above_ma60, stronger_than_market, obv_uptrend, cci_momentum, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="2" t="n">
-        <v>6291</v>
+        <v>6279</v>
       </c>
       <c r="B61" s="2" t="inlineStr">
         <is>
-          <t>沛亨</t>
+          <t>胡連</t>
         </is>
       </c>
       <c r="C61" s="2" t="n">
         <v/>
       </c>
       <c r="D61" s="2" t="n">
-        <v>618.4533524331326</v>
+        <v>624.1513423914423</v>
       </c>
       <c r="E61" s="2" t="n">
-        <v>563</v>
+        <v>120</v>
       </c>
       <c r="F61" s="2" t="inlineStr">
         <is>
@@ -3679,49 +3679,49 @@
         <v>0</v>
       </c>
       <c r="H61" s="2" t="n">
-        <v>52.65126228651362</v>
+        <v>52.52891393379767</v>
       </c>
       <c r="I61" s="2" t="n">
-        <v>19.46637208983243</v>
+        <v>18.79887470791074</v>
       </c>
       <c r="J61" s="2" t="n">
-        <v>0.7216998127345161</v>
+        <v>0.3956414609622081</v>
       </c>
       <c r="K61" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L61" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M61" s="2" t="n">
         <v>-1</v>
       </c>
       <c r="N61" s="2" t="n">
-        <v>-5.529840541615783</v>
+        <v>-0.2960388297891239</v>
       </c>
       <c r="O61" s="2" t="inlineStr">
         <is>
-          <t>above_ema60, ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, stronger_than_market, obv_uptrend, above_ichimoku_cloud</t>
+          <t>above_ema60, market_above_ma60, avoid_chase, liquidity_ok, stronger_than_market, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="n">
-        <v>6283</v>
+        <v>6291</v>
       </c>
       <c r="B62" s="2" t="inlineStr">
         <is>
-          <t>淳安</t>
+          <t>沛亨</t>
         </is>
       </c>
       <c r="C62" s="2" t="n">
         <v/>
       </c>
       <c r="D62" s="2" t="n">
-        <v>617.3954084251953</v>
+        <v>618.4533524331326</v>
       </c>
       <c r="E62" s="2" t="n">
-        <v>24.3</v>
+        <v>563</v>
       </c>
       <c r="F62" s="2" t="inlineStr">
         <is>
@@ -3732,49 +3732,49 @@
         <v>0</v>
       </c>
       <c r="H62" s="2" t="n">
-        <v>51.36454314919617</v>
+        <v>52.65126228651362</v>
       </c>
       <c r="I62" s="2" t="n">
-        <v>16.18055759139992</v>
+        <v>19.46637208983243</v>
       </c>
       <c r="J62" s="2" t="n">
-        <v>0.4759086571158815</v>
+        <v>0.7216998127345161</v>
       </c>
       <c r="K62" s="2" t="n">
         <v>1</v>
       </c>
       <c r="L62" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M62" s="2" t="n">
         <v>-1</v>
       </c>
       <c r="N62" s="2" t="n">
-        <v>-0.0589830218632357</v>
+        <v>-5.529840541615783</v>
       </c>
       <c r="O62" s="2" t="inlineStr">
         <is>
-          <t>above_ema60, ema60_gt_ema120, market_above_ma60, avoid_chase, stronger_than_market, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
+          <t>above_ema60, ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, stronger_than_market, obv_uptrend, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="2" t="n">
-        <v>6164</v>
+        <v>6283</v>
       </c>
       <c r="B63" s="2" t="inlineStr">
         <is>
-          <t>華興</t>
+          <t>淳安</t>
         </is>
       </c>
       <c r="C63" s="2" t="n">
         <v/>
       </c>
       <c r="D63" s="2" t="n">
-        <v>613.492500196535</v>
+        <v>617.3954084251953</v>
       </c>
       <c r="E63" s="2" t="n">
-        <v>13.55</v>
+        <v>24.3</v>
       </c>
       <c r="F63" s="2" t="inlineStr">
         <is>
@@ -3785,16 +3785,16 @@
         <v>0</v>
       </c>
       <c r="H63" s="2" t="n">
-        <v>58.51236649114365</v>
+        <v>51.36454314919617</v>
       </c>
       <c r="I63" s="2" t="n">
-        <v>22.39231391968946</v>
+        <v>16.18055759139992</v>
       </c>
       <c r="J63" s="2" t="n">
-        <v>0.9538763345562988</v>
+        <v>0.4759086571158815</v>
       </c>
       <c r="K63" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L63" s="2" t="n">
         <v>0</v>
@@ -3803,31 +3803,31 @@
         <v>-1</v>
       </c>
       <c r="N63" s="2" t="n">
-        <v>0.0796354767884002</v>
+        <v>-0.0589830218632357</v>
       </c>
       <c r="O63" s="2" t="inlineStr">
         <is>
-          <t>above_ema60, ema60_gt_ema120, rsi_strong, market_above_ma60, adx_trending, stronger_than_market, mfi_strong, above_ichimoku_cloud</t>
+          <t>above_ema60, ema60_gt_ema120, market_above_ma60, avoid_chase, stronger_than_market, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="n">
-        <v>6290</v>
+        <v>6164</v>
       </c>
       <c r="B64" s="2" t="inlineStr">
         <is>
-          <t>良維</t>
+          <t>華興</t>
         </is>
       </c>
       <c r="C64" s="2" t="n">
         <v/>
       </c>
       <c r="D64" s="2" t="n">
-        <v>608.2151014073778</v>
+        <v>613.492500196535</v>
       </c>
       <c r="E64" s="2" t="n">
-        <v>306</v>
+        <v>13.55</v>
       </c>
       <c r="F64" s="2" t="inlineStr">
         <is>
@@ -3838,13 +3838,13 @@
         <v>0</v>
       </c>
       <c r="H64" s="2" t="n">
-        <v>49.24655293432787</v>
+        <v>58.51236649114365</v>
       </c>
       <c r="I64" s="2" t="n">
-        <v>14.9014048099975</v>
+        <v>22.39231391968946</v>
       </c>
       <c r="J64" s="2" t="n">
-        <v>0.773187358105673</v>
+        <v>0.9538763345562988</v>
       </c>
       <c r="K64" s="2" t="n">
         <v>0</v>
@@ -3856,31 +3856,31 @@
         <v>-1</v>
       </c>
       <c r="N64" s="2" t="n">
-        <v>-3.914009715755391</v>
+        <v>0.0796354767884002</v>
       </c>
       <c r="O64" s="2" t="inlineStr">
         <is>
-          <t>above_ema60, ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, stronger_than_market, obv_uptrend, above_ichimoku_cloud</t>
+          <t>above_ema60, ema60_gt_ema120, rsi_strong, market_above_ma60, adx_trending, stronger_than_market, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="2" t="n">
-        <v>6206</v>
+        <v>6290</v>
       </c>
       <c r="B65" s="2" t="inlineStr">
         <is>
-          <t>飛捷</t>
+          <t>良維</t>
         </is>
       </c>
       <c r="C65" s="2" t="n">
         <v/>
       </c>
       <c r="D65" s="2" t="n">
-        <v>606.8278620055498</v>
+        <v>608.2151014073778</v>
       </c>
       <c r="E65" s="2" t="n">
-        <v>130.5</v>
+        <v>306</v>
       </c>
       <c r="F65" s="2" t="inlineStr">
         <is>
@@ -3891,13 +3891,13 @@
         <v>0</v>
       </c>
       <c r="H65" s="2" t="n">
-        <v>47.86399578780711</v>
+        <v>49.24655293432787</v>
       </c>
       <c r="I65" s="2" t="n">
-        <v>18.68983197969632</v>
+        <v>14.9014048099975</v>
       </c>
       <c r="J65" s="2" t="n">
-        <v>0.3983740891451739</v>
+        <v>0.773187358105673</v>
       </c>
       <c r="K65" s="2" t="n">
         <v>0</v>
@@ -3909,31 +3909,31 @@
         <v>-1</v>
       </c>
       <c r="N65" s="2" t="n">
-        <v>-1.340635324985543</v>
+        <v>-3.914009715755391</v>
       </c>
       <c r="O65" s="2" t="inlineStr">
         <is>
-          <t>above_ema60, ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, stronger_than_market, kd_golden_cross, above_ichimoku_cloud</t>
+          <t>above_ema60, ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, stronger_than_market, obv_uptrend, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="2" t="n">
-        <v>6227</v>
+        <v>6206</v>
       </c>
       <c r="B66" s="2" t="inlineStr">
         <is>
-          <t>茂綸</t>
+          <t>飛捷</t>
         </is>
       </c>
       <c r="C66" s="2" t="n">
         <v/>
       </c>
       <c r="D66" s="2" t="n">
-        <v>598.9668882619068</v>
+        <v>606.8278620055498</v>
       </c>
       <c r="E66" s="2" t="n">
-        <v>119.5</v>
+        <v>130.5</v>
       </c>
       <c r="F66" s="2" t="inlineStr">
         <is>
@@ -3944,13 +3944,13 @@
         <v>0</v>
       </c>
       <c r="H66" s="2" t="n">
-        <v>47.01629718231956</v>
+        <v>47.86399578780711</v>
       </c>
       <c r="I66" s="2" t="n">
-        <v>21.2209080974055</v>
+        <v>18.68983197969632</v>
       </c>
       <c r="J66" s="2" t="n">
-        <v>0.219147797795077</v>
+        <v>0.3983740891451739</v>
       </c>
       <c r="K66" s="2" t="n">
         <v>0</v>
@@ -3962,31 +3962,31 @@
         <v>-1</v>
       </c>
       <c r="N66" s="2" t="n">
-        <v>-2.214509177971088</v>
+        <v>-1.340635324985543</v>
       </c>
       <c r="O66" s="2" t="inlineStr">
         <is>
-          <t>above_ema60, ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, kd_golden_cross, above_ichimoku_cloud</t>
+          <t>above_ema60, ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, stronger_than_market, kd_golden_cross, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="2" t="n">
-        <v>6278</v>
+        <v>6227</v>
       </c>
       <c r="B67" s="2" t="inlineStr">
         <is>
-          <t>台表科</t>
+          <t>茂綸</t>
         </is>
       </c>
       <c r="C67" s="2" t="n">
         <v/>
       </c>
       <c r="D67" s="2" t="n">
-        <v>581.9839660814002</v>
+        <v>598.9668882619068</v>
       </c>
       <c r="E67" s="2" t="n">
-        <v>201.5</v>
+        <v>119.5</v>
       </c>
       <c r="F67" s="2" t="inlineStr">
         <is>
@@ -3997,16 +3997,16 @@
         <v>0</v>
       </c>
       <c r="H67" s="2" t="n">
-        <v>48.81223555988845</v>
+        <v>47.01629718231956</v>
       </c>
       <c r="I67" s="2" t="n">
-        <v>21.19336588985524</v>
+        <v>21.2209080974055</v>
       </c>
       <c r="J67" s="2" t="n">
-        <v>0.3625691030812945</v>
+        <v>0.219147797795077</v>
       </c>
       <c r="K67" s="2" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="L67" s="2" t="n">
         <v>0</v>
@@ -4015,31 +4015,31 @@
         <v>-1</v>
       </c>
       <c r="N67" s="2" t="n">
-        <v>-2.307613214695454</v>
+        <v>-2.214509177971088</v>
       </c>
       <c r="O67" s="2" t="inlineStr">
         <is>
-          <t>above_ema60, ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, foreign_buy_3d, adx_trending, above_ichimoku_cloud</t>
+          <t>above_ema60, ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, kd_golden_cross, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="2" t="n">
-        <v>6185</v>
+        <v>6278</v>
       </c>
       <c r="B68" s="2" t="inlineStr">
         <is>
-          <t>幃翔</t>
+          <t>台表科</t>
         </is>
       </c>
       <c r="C68" s="2" t="n">
         <v/>
       </c>
       <c r="D68" s="2" t="n">
-        <v>581.4901784832014</v>
+        <v>581.9839660814002</v>
       </c>
       <c r="E68" s="2" t="n">
-        <v>14.4</v>
+        <v>201.5</v>
       </c>
       <c r="F68" s="2" t="inlineStr">
         <is>
@@ -4050,16 +4050,16 @@
         <v>0</v>
       </c>
       <c r="H68" s="2" t="n">
-        <v>54.54724712679436</v>
+        <v>48.81223555988845</v>
       </c>
       <c r="I68" s="2" t="n">
-        <v>16.69905483705111</v>
+        <v>21.19336588985524</v>
       </c>
       <c r="J68" s="2" t="n">
-        <v>0.7622340525812163</v>
+        <v>0.3625691030812945</v>
       </c>
       <c r="K68" s="2" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="L68" s="2" t="n">
         <v>0</v>
@@ -4068,31 +4068,31 @@
         <v>-1</v>
       </c>
       <c r="N68" s="2" t="n">
-        <v>0.0267498064798663</v>
+        <v>-2.307613214695454</v>
       </c>
       <c r="O68" s="2" t="inlineStr">
         <is>
-          <t>above_ema60, market_above_ma60, avoid_chase, stronger_than_market, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
+          <t>above_ema60, ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, foreign_buy_3d, adx_trending, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" s="2" t="n">
-        <v>6214</v>
+        <v>6185</v>
       </c>
       <c r="B69" s="2" t="inlineStr">
         <is>
-          <t>精誠</t>
+          <t>幃翔</t>
         </is>
       </c>
       <c r="C69" s="2" t="n">
         <v/>
       </c>
       <c r="D69" s="2" t="n">
-        <v>562.0607874575886</v>
+        <v>581.4901784832014</v>
       </c>
       <c r="E69" s="2" t="n">
-        <v>131</v>
+        <v>14.4</v>
       </c>
       <c r="F69" s="2" t="inlineStr">
         <is>
@@ -4103,16 +4103,16 @@
         <v>0</v>
       </c>
       <c r="H69" s="2" t="n">
-        <v>42.72561918602374</v>
+        <v>54.54724712679436</v>
       </c>
       <c r="I69" s="2" t="n">
-        <v>20.343003106727</v>
+        <v>16.69905483705111</v>
       </c>
       <c r="J69" s="2" t="n">
-        <v>0.4636911918388798</v>
+        <v>0.7622340525812163</v>
       </c>
       <c r="K69" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L69" s="2" t="n">
         <v>0</v>
@@ -4121,31 +4121,31 @@
         <v>-1</v>
       </c>
       <c r="N69" s="2" t="n">
-        <v>-2.148160308433721</v>
+        <v>0.0267498064798663</v>
       </c>
       <c r="O69" s="2" t="inlineStr">
         <is>
-          <t>above_ema60, ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, kd_golden_cross, above_ichimoku_cloud</t>
+          <t>above_ema60, market_above_ma60, avoid_chase, stronger_than_market, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" s="2" t="n">
-        <v>6470</v>
+        <v>6214</v>
       </c>
       <c r="B70" s="2" t="inlineStr">
         <is>
-          <t>宇智</t>
+          <t>精誠</t>
         </is>
       </c>
       <c r="C70" s="2" t="n">
         <v/>
       </c>
       <c r="D70" s="2" t="n">
-        <v>552.6694677354241</v>
+        <v>562.0607874575886</v>
       </c>
       <c r="E70" s="2" t="n">
-        <v>49.6</v>
+        <v>131</v>
       </c>
       <c r="F70" s="2" t="inlineStr">
         <is>
@@ -4156,16 +4156,16 @@
         <v>0</v>
       </c>
       <c r="H70" s="2" t="n">
-        <v>54.76843696846535</v>
+        <v>42.72561918602374</v>
       </c>
       <c r="I70" s="2" t="n">
-        <v>15.72228211520844</v>
+        <v>20.343003106727</v>
       </c>
       <c r="J70" s="2" t="n">
-        <v>0.5712810205733746</v>
+        <v>0.4636911918388798</v>
       </c>
       <c r="K70" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L70" s="2" t="n">
         <v>0</v>
@@ -4174,31 +4174,31 @@
         <v>-1</v>
       </c>
       <c r="N70" s="2" t="n">
-        <v>0.0364262059958838</v>
+        <v>-2.148160308433721</v>
       </c>
       <c r="O70" s="2" t="inlineStr">
         <is>
-          <t>above_ema60, ema60_gt_ema120, market_above_ma60, avoid_chase, stronger_than_market, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
+          <t>above_ema60, ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, kd_golden_cross, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" s="2" t="n">
-        <v>6456</v>
+        <v>6470</v>
       </c>
       <c r="B71" s="2" t="inlineStr">
         <is>
-          <t>GIS-KY</t>
+          <t>宇智</t>
         </is>
       </c>
       <c r="C71" s="2" t="n">
         <v/>
       </c>
       <c r="D71" s="2" t="n">
-        <v>552.5587470367974</v>
+        <v>552.6694677354241</v>
       </c>
       <c r="E71" s="2" t="n">
-        <v>73.7</v>
+        <v>49.6</v>
       </c>
       <c r="F71" s="2" t="inlineStr">
         <is>
@@ -4209,16 +4209,16 @@
         <v>0</v>
       </c>
       <c r="H71" s="2" t="n">
-        <v>48.88201080208466</v>
+        <v>54.76843696846535</v>
       </c>
       <c r="I71" s="2" t="n">
-        <v>12.07473807590211</v>
+        <v>15.72228211520844</v>
       </c>
       <c r="J71" s="2" t="n">
-        <v>0.4068350072930159</v>
+        <v>0.5712810205733746</v>
       </c>
       <c r="K71" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L71" s="2" t="n">
         <v>0</v>
@@ -4227,31 +4227,31 @@
         <v>-1</v>
       </c>
       <c r="N71" s="2" t="n">
-        <v>-0.6636894251423329</v>
+        <v>0.0364262059958838</v>
       </c>
       <c r="O71" s="2" t="inlineStr">
         <is>
-          <t>above_ema60, ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, stronger_than_market, kd_golden_cross, above_ichimoku_cloud</t>
+          <t>above_ema60, ema60_gt_ema120, market_above_ma60, avoid_chase, stronger_than_market, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" s="2" t="n">
-        <v>6261</v>
+        <v>6456</v>
       </c>
       <c r="B72" s="2" t="inlineStr">
         <is>
-          <t>久元</t>
+          <t>GIS-KY</t>
         </is>
       </c>
       <c r="C72" s="2" t="n">
         <v/>
       </c>
       <c r="D72" s="2" t="n">
-        <v>551.7809623922324</v>
+        <v>552.5587470367974</v>
       </c>
       <c r="E72" s="2" t="n">
-        <v>99.5</v>
+        <v>73.7</v>
       </c>
       <c r="F72" s="2" t="inlineStr">
         <is>
@@ -4262,13 +4262,13 @@
         <v>0</v>
       </c>
       <c r="H72" s="2" t="n">
-        <v>45.78498916561272</v>
+        <v>48.88201080208466</v>
       </c>
       <c r="I72" s="2" t="n">
-        <v>21.60031634479152</v>
+        <v>12.07473807590211</v>
       </c>
       <c r="J72" s="2" t="n">
-        <v>0.4903960202587745</v>
+        <v>0.4068350072930159</v>
       </c>
       <c r="K72" s="2" t="n">
         <v>0</v>
@@ -4280,31 +4280,31 @@
         <v>-1</v>
       </c>
       <c r="N72" s="2" t="n">
-        <v>-0.642360515217602</v>
+        <v>-0.6636894251423329</v>
       </c>
       <c r="O72" s="2" t="inlineStr">
         <is>
-          <t>above_ema60, ema60_gt_ema120, market_above_ma60, liquidity_ok, adx_trending, stronger_than_market, kd_golden_cross</t>
+          <t>above_ema60, ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, stronger_than_market, kd_golden_cross, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" s="2" t="n">
-        <v>6177</v>
+        <v>6261</v>
       </c>
       <c r="B73" s="2" t="inlineStr">
         <is>
-          <t>達麗</t>
+          <t>久元</t>
         </is>
       </c>
       <c r="C73" s="2" t="n">
         <v/>
       </c>
       <c r="D73" s="2" t="n">
-        <v>540.0420210490283</v>
+        <v>551.7809623922324</v>
       </c>
       <c r="E73" s="2" t="n">
-        <v>46.1</v>
+        <v>99.5</v>
       </c>
       <c r="F73" s="2" t="inlineStr">
         <is>
@@ -4315,16 +4315,16 @@
         <v>0</v>
       </c>
       <c r="H73" s="2" t="n">
-        <v>50.8014115782721</v>
+        <v>45.78498916561272</v>
       </c>
       <c r="I73" s="2" t="n">
-        <v>22.65458245793009</v>
+        <v>21.60031634479152</v>
       </c>
       <c r="J73" s="2" t="n">
-        <v>0.3780711053934805</v>
+        <v>0.4903960202587745</v>
       </c>
       <c r="K73" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L73" s="2" t="n">
         <v>0</v>
@@ -4333,31 +4333,31 @@
         <v>-1</v>
       </c>
       <c r="N73" s="2" t="n">
-        <v>0.0981701661587394</v>
+        <v>-0.642360515217602</v>
       </c>
       <c r="O73" s="2" t="inlineStr">
         <is>
-          <t>above_ema60, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, obv_uptrend, mfi_strong</t>
+          <t>above_ema60, ema60_gt_ema120, market_above_ma60, liquidity_ok, adx_trending, stronger_than_market, kd_golden_cross</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" s="2" t="n">
-        <v>6417</v>
+        <v>6177</v>
       </c>
       <c r="B74" s="2" t="inlineStr">
         <is>
-          <t>韋僑</t>
+          <t>達麗</t>
         </is>
       </c>
       <c r="C74" s="2" t="n">
         <v/>
       </c>
       <c r="D74" s="2" t="n">
-        <v>522.7944502793713</v>
+        <v>540.0420210490283</v>
       </c>
       <c r="E74" s="2" t="n">
-        <v>130.5</v>
+        <v>46.1</v>
       </c>
       <c r="F74" s="2" t="inlineStr">
         <is>
@@ -4368,13 +4368,13 @@
         <v>0</v>
       </c>
       <c r="H74" s="2" t="n">
-        <v>47.30507523607982</v>
+        <v>50.8014115782721</v>
       </c>
       <c r="I74" s="2" t="n">
-        <v>15.79515073734375</v>
+        <v>22.65458245793009</v>
       </c>
       <c r="J74" s="2" t="n">
-        <v>0.2569311176874689</v>
+        <v>0.3780711053934805</v>
       </c>
       <c r="K74" s="2" t="n">
         <v>1</v>
@@ -4386,31 +4386,31 @@
         <v>-1</v>
       </c>
       <c r="N74" s="2" t="n">
-        <v>-1.308526632843335</v>
+        <v>0.0981701661587394</v>
       </c>
       <c r="O74" s="2" t="inlineStr">
         <is>
-          <t>above_ema60, ema60_gt_ema120, market_above_ma60, avoid_chase, stronger_than_market, kd_golden_cross, obv_uptrend</t>
+          <t>above_ema60, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" s="2" t="n">
-        <v>6285</v>
+        <v>6417</v>
       </c>
       <c r="B75" s="2" t="inlineStr">
         <is>
-          <t>啟碁</t>
+          <t>韋僑</t>
         </is>
       </c>
       <c r="C75" s="2" t="n">
         <v/>
       </c>
       <c r="D75" s="2" t="n">
-        <v>510.1451212517223</v>
+        <v>522.7944502793713</v>
       </c>
       <c r="E75" s="2" t="n">
-        <v>255</v>
+        <v>130.5</v>
       </c>
       <c r="F75" s="2" t="inlineStr">
         <is>
@@ -4421,13 +4421,13 @@
         <v>0</v>
       </c>
       <c r="H75" s="2" t="n">
-        <v>41.33689987603705</v>
+        <v>47.30507523607982</v>
       </c>
       <c r="I75" s="2" t="n">
-        <v>21.18189972570445</v>
+        <v>15.79515073734375</v>
       </c>
       <c r="J75" s="2" t="n">
-        <v>0.5045712299396238</v>
+        <v>0.2569311176874689</v>
       </c>
       <c r="K75" s="2" t="n">
         <v>1</v>
@@ -4439,31 +4439,31 @@
         <v>-1</v>
       </c>
       <c r="N75" s="2" t="n">
-        <v>-5.289547502302751</v>
+        <v>-1.308526632843335</v>
       </c>
       <c r="O75" s="2" t="inlineStr">
         <is>
-          <t>above_ema60, ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, above_ichimoku_cloud</t>
+          <t>above_ema60, ema60_gt_ema120, market_above_ma60, avoid_chase, stronger_than_market, kd_golden_cross, obv_uptrend</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" s="2" t="n">
-        <v>6192</v>
+        <v>6285</v>
       </c>
       <c r="B76" s="2" t="inlineStr">
         <is>
-          <t>巨路</t>
+          <t>啟碁</t>
         </is>
       </c>
       <c r="C76" s="2" t="n">
         <v/>
       </c>
       <c r="D76" s="2" t="n">
-        <v>489.2796672529384</v>
+        <v>510.1451212517223</v>
       </c>
       <c r="E76" s="2" t="n">
-        <v>121</v>
+        <v>255</v>
       </c>
       <c r="F76" s="2" t="inlineStr">
         <is>
@@ -4474,16 +4474,16 @@
         <v>0</v>
       </c>
       <c r="H76" s="2" t="n">
-        <v>46.17765093034743</v>
+        <v>41.33689987603705</v>
       </c>
       <c r="I76" s="2" t="n">
-        <v>24.21183979122784</v>
+        <v>21.18189972570445</v>
       </c>
       <c r="J76" s="2" t="n">
-        <v>1.624726574447245</v>
+        <v>0.5045712299396238</v>
       </c>
       <c r="K76" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L76" s="2" t="n">
         <v>0</v>
@@ -4492,31 +4492,31 @@
         <v>-1</v>
       </c>
       <c r="N76" s="2" t="n">
-        <v>-0.5733924992416002</v>
+        <v>-5.289547502302751</v>
       </c>
       <c r="O76" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, volume_break, market_above_ma60, avoid_chase, adx_trending, stronger_than_market, obv_uptrend</t>
+          <t>above_ema60, ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" s="2" t="n">
-        <v>6438</v>
+        <v>6192</v>
       </c>
       <c r="B77" s="2" t="inlineStr">
         <is>
-          <t>迅得</t>
+          <t>巨路</t>
         </is>
       </c>
       <c r="C77" s="2" t="n">
         <v/>
       </c>
       <c r="D77" s="2" t="n">
-        <v>487.7375864056355</v>
+        <v>489.2796672529384</v>
       </c>
       <c r="E77" s="2" t="n">
-        <v>152.5</v>
+        <v>121</v>
       </c>
       <c r="F77" s="2" t="inlineStr">
         <is>
@@ -4527,16 +4527,16 @@
         <v>0</v>
       </c>
       <c r="H77" s="2" t="n">
-        <v>42.8205984927579</v>
+        <v>46.17765093034743</v>
       </c>
       <c r="I77" s="2" t="n">
-        <v>24.82227006488733</v>
+        <v>24.21183979122784</v>
       </c>
       <c r="J77" s="2" t="n">
-        <v>0.537052633629062</v>
+        <v>1.624726574447245</v>
       </c>
       <c r="K77" s="2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="L77" s="2" t="n">
         <v>0</v>
@@ -4545,31 +4545,31 @@
         <v>-1</v>
       </c>
       <c r="N77" s="2" t="n">
-        <v>0.5716184354181273</v>
+        <v>-0.5733924992416002</v>
       </c>
       <c r="O77" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, stronger_than_market</t>
+          <t>ema60_gt_ema120, volume_break, market_above_ma60, avoid_chase, adx_trending, stronger_than_market, obv_uptrend</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" s="2" t="n">
-        <v>6176</v>
+        <v>6438</v>
       </c>
       <c r="B78" s="2" t="inlineStr">
         <is>
-          <t>瑞儀</t>
+          <t>迅得</t>
         </is>
       </c>
       <c r="C78" s="2" t="n">
         <v/>
       </c>
       <c r="D78" s="2" t="n">
-        <v>487.3985044975937</v>
+        <v>487.7375864056355</v>
       </c>
       <c r="E78" s="2" t="n">
-        <v>90.2</v>
+        <v>152.5</v>
       </c>
       <c r="F78" s="2" t="inlineStr">
         <is>
@@ -4580,16 +4580,16 @@
         <v>0</v>
       </c>
       <c r="H78" s="2" t="n">
-        <v>38.83593112846242</v>
+        <v>42.8205984927579</v>
       </c>
       <c r="I78" s="2" t="n">
-        <v>25.72802949137787</v>
+        <v>24.82227006488733</v>
       </c>
       <c r="J78" s="2" t="n">
-        <v>0.8061030408440726</v>
+        <v>0.537052633629062</v>
       </c>
       <c r="K78" s="2" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L78" s="2" t="n">
         <v>0</v>
@@ -4598,31 +4598,31 @@
         <v>-1</v>
       </c>
       <c r="N78" s="2" t="n">
-        <v>-0.463686749658716</v>
+        <v>0.5716184354181273</v>
       </c>
       <c r="O78" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, liquidity_ok, foreign_buy_3d, adx_trending, stronger_than_market</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, stronger_than_market</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" s="2" t="n">
-        <v>6277</v>
+        <v>6176</v>
       </c>
       <c r="B79" s="2" t="inlineStr">
         <is>
-          <t>宏正</t>
+          <t>瑞儀</t>
         </is>
       </c>
       <c r="C79" s="2" t="n">
         <v/>
       </c>
       <c r="D79" s="2" t="n">
-        <v>474.1165154704151</v>
+        <v>487.3985044975937</v>
       </c>
       <c r="E79" s="2" t="n">
-        <v>71.2</v>
+        <v>90.2</v>
       </c>
       <c r="F79" s="2" t="inlineStr">
         <is>
@@ -4633,16 +4633,16 @@
         <v>0</v>
       </c>
       <c r="H79" s="2" t="n">
-        <v>40.24900314203754</v>
+        <v>38.83593112846242</v>
       </c>
       <c r="I79" s="2" t="n">
-        <v>30.66911393492165</v>
+        <v>25.72802949137787</v>
       </c>
       <c r="J79" s="2" t="n">
-        <v>0.2985930576163298</v>
+        <v>0.8061030408440726</v>
       </c>
       <c r="K79" s="2" t="n">
-        <v>13</v>
+        <v>3</v>
       </c>
       <c r="L79" s="2" t="n">
         <v>0</v>
@@ -4651,31 +4651,31 @@
         <v>-1</v>
       </c>
       <c r="N79" s="2" t="n">
-        <v>-0.7538337713015097</v>
+        <v>-0.463686749658716</v>
       </c>
       <c r="O79" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, foreign_buy_3d, adx_trending, kd_golden_cross</t>
+          <t>market_above_ma60, avoid_chase, liquidity_ok, foreign_buy_3d, adx_trending, stronger_than_market</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" s="2" t="n">
-        <v>6442</v>
+        <v>6277</v>
       </c>
       <c r="B80" s="2" t="inlineStr">
         <is>
-          <t>光聖</t>
+          <t>宏正</t>
         </is>
       </c>
       <c r="C80" s="2" t="n">
         <v/>
       </c>
       <c r="D80" s="2" t="n">
-        <v>463.6972278953296</v>
+        <v>474.1165154704151</v>
       </c>
       <c r="E80" s="2" t="n">
-        <v>1935</v>
+        <v>71.2</v>
       </c>
       <c r="F80" s="2" t="inlineStr">
         <is>
@@ -4686,49 +4686,49 @@
         <v>0</v>
       </c>
       <c r="H80" s="2" t="n">
-        <v>49.33653996083048</v>
+        <v>40.24900314203754</v>
       </c>
       <c r="I80" s="2" t="n">
-        <v>11.7534635991202</v>
+        <v>30.66911393492165</v>
       </c>
       <c r="J80" s="2" t="n">
-        <v>0.8638930083981431</v>
+        <v>0.2985930576163298</v>
       </c>
       <c r="K80" s="2" t="n">
-        <v>0</v>
+        <v>13</v>
       </c>
       <c r="L80" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M80" s="2" t="n">
         <v>-1</v>
       </c>
       <c r="N80" s="2" t="n">
-        <v>4.678750429020333</v>
+        <v>-0.7538337713015097</v>
       </c>
       <c r="O80" s="2" t="inlineStr">
         <is>
-          <t>above_ema60, ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, stronger_than_market</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, foreign_buy_3d, adx_trending, kd_golden_cross</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" s="2" t="n">
-        <v>6418</v>
+        <v>6442</v>
       </c>
       <c r="B81" s="2" t="inlineStr">
         <is>
-          <t>詠昇</t>
+          <t>光聖</t>
         </is>
       </c>
       <c r="C81" s="2" t="n">
         <v/>
       </c>
       <c r="D81" s="2" t="n">
-        <v>454.2989478058981</v>
+        <v>463.6972278953296</v>
       </c>
       <c r="E81" s="2" t="n">
-        <v>31.2</v>
+        <v>1935</v>
       </c>
       <c r="F81" s="2" t="inlineStr">
         <is>
@@ -4739,49 +4739,49 @@
         <v>0</v>
       </c>
       <c r="H81" s="2" t="n">
-        <v>47.80023164365148</v>
+        <v>49.33653996083048</v>
       </c>
       <c r="I81" s="2" t="n">
-        <v>23.6883472518325</v>
+        <v>11.7534635991202</v>
       </c>
       <c r="J81" s="2" t="n">
-        <v>0.4001195229118434</v>
+        <v>0.8638930083981431</v>
       </c>
       <c r="K81" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L81" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="L81" s="2" t="n">
-        <v>0</v>
-      </c>
       <c r="M81" s="2" t="n">
         <v>-1</v>
       </c>
       <c r="N81" s="2" t="n">
-        <v>-0.0919654863080669</v>
+        <v>4.678750429020333</v>
       </c>
       <c r="O81" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, adx_trending, kd_golden_cross, obv_uptrend, mfi_strong</t>
+          <t>above_ema60, ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, stronger_than_market</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" s="2" t="n">
-        <v>6198</v>
+        <v>6418</v>
       </c>
       <c r="B82" s="2" t="inlineStr">
         <is>
-          <t>瑞築</t>
+          <t>詠昇</t>
         </is>
       </c>
       <c r="C82" s="2" t="n">
         <v/>
       </c>
       <c r="D82" s="2" t="n">
-        <v>442.2535819448876</v>
+        <v>454.2989478058981</v>
       </c>
       <c r="E82" s="2" t="n">
-        <v>20.65</v>
+        <v>31.2</v>
       </c>
       <c r="F82" s="2" t="inlineStr">
         <is>
@@ -4792,16 +4792,16 @@
         <v>0</v>
       </c>
       <c r="H82" s="2" t="n">
-        <v>51.20636424249206</v>
+        <v>47.80023164365148</v>
       </c>
       <c r="I82" s="2" t="n">
-        <v>7.684849923736959</v>
+        <v>23.6883472518325</v>
       </c>
       <c r="J82" s="2" t="n">
-        <v>0.4389591220817558</v>
+        <v>0.4001195229118434</v>
       </c>
       <c r="K82" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L82" s="2" t="n">
         <v>0</v>
@@ -4810,31 +4810,31 @@
         <v>-1</v>
       </c>
       <c r="N82" s="2" t="n">
-        <v>0.3544815421059192</v>
+        <v>-0.0919654863080669</v>
       </c>
       <c r="O82" s="2" t="inlineStr">
         <is>
-          <t>above_ema60, market_above_ma60, avoid_chase, kd_golden_cross, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
+          <t>market_above_ma60, avoid_chase, adx_trending, kd_golden_cross, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" s="2" t="n">
-        <v>6216</v>
+        <v>6198</v>
       </c>
       <c r="B83" s="2" t="inlineStr">
         <is>
-          <t>居易</t>
+          <t>瑞築</t>
         </is>
       </c>
       <c r="C83" s="2" t="n">
         <v/>
       </c>
       <c r="D83" s="2" t="n">
-        <v>438.5822687127638</v>
+        <v>442.2535819448876</v>
       </c>
       <c r="E83" s="2" t="n">
-        <v>23.2</v>
+        <v>20.65</v>
       </c>
       <c r="F83" s="2" t="inlineStr">
         <is>
@@ -4845,16 +4845,16 @@
         <v>0</v>
       </c>
       <c r="H83" s="2" t="n">
-        <v>51.66793492835279</v>
+        <v>51.20636424249206</v>
       </c>
       <c r="I83" s="2" t="n">
-        <v>15.86328745697326</v>
+        <v>7.684849923736959</v>
       </c>
       <c r="J83" s="2" t="n">
-        <v>1.242233021158403</v>
+        <v>0.4389591220817558</v>
       </c>
       <c r="K83" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L83" s="2" t="n">
         <v>0</v>
@@ -4863,31 +4863,31 @@
         <v>-1</v>
       </c>
       <c r="N83" s="2" t="n">
-        <v>0.08062650583180769</v>
+        <v>0.3544815421059192</v>
       </c>
       <c r="O83" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, stronger_than_market, kd_golden_cross, obv_uptrend, mfi_strong</t>
+          <t>above_ema60, market_above_ma60, avoid_chase, kd_golden_cross, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" s="2" t="n">
-        <v>6244</v>
+        <v>6216</v>
       </c>
       <c r="B84" s="2" t="inlineStr">
         <is>
-          <t>茂迪</t>
+          <t>居易</t>
         </is>
       </c>
       <c r="C84" s="2" t="n">
         <v/>
       </c>
       <c r="D84" s="2" t="n">
-        <v>426.9241965200596</v>
+        <v>438.5822687127638</v>
       </c>
       <c r="E84" s="2" t="n">
-        <v>27.9</v>
+        <v>23.2</v>
       </c>
       <c r="F84" s="2" t="inlineStr">
         <is>
@@ -4898,16 +4898,16 @@
         <v>0</v>
       </c>
       <c r="H84" s="2" t="n">
-        <v>44.81433877013381</v>
+        <v>51.66793492835279</v>
       </c>
       <c r="I84" s="2" t="n">
-        <v>18.39286373204455</v>
+        <v>15.86328745697326</v>
       </c>
       <c r="J84" s="2" t="n">
-        <v>0.398609953485921</v>
+        <v>1.242233021158403</v>
       </c>
       <c r="K84" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L84" s="2" t="n">
         <v>0</v>
@@ -4916,31 +4916,31 @@
         <v>-1</v>
       </c>
       <c r="N84" s="2" t="n">
-        <v>-0.3031502392603908</v>
+        <v>0.08062650583180769</v>
       </c>
       <c r="O84" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, obv_uptrend, mfi_strong</t>
+          <t>market_above_ma60, avoid_chase, stronger_than_market, kd_golden_cross, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" s="2" t="n">
-        <v>6412</v>
+        <v>6244</v>
       </c>
       <c r="B85" s="2" t="inlineStr">
         <is>
-          <t>群電</t>
+          <t>茂迪</t>
         </is>
       </c>
       <c r="C85" s="2" t="n">
         <v/>
       </c>
       <c r="D85" s="2" t="n">
-        <v>423.3048338069732</v>
+        <v>426.9241965200596</v>
       </c>
       <c r="E85" s="2" t="n">
-        <v>93.09999999999999</v>
+        <v>27.9</v>
       </c>
       <c r="F85" s="2" t="inlineStr">
         <is>
@@ -4951,13 +4951,13 @@
         <v>0</v>
       </c>
       <c r="H85" s="2" t="n">
-        <v>49.05189400226433</v>
+        <v>44.81433877013381</v>
       </c>
       <c r="I85" s="2" t="n">
-        <v>19.53005845025127</v>
+        <v>18.39286373204455</v>
       </c>
       <c r="J85" s="2" t="n">
-        <v>0.5443375335334363</v>
+        <v>0.398609953485921</v>
       </c>
       <c r="K85" s="2" t="n">
         <v>0</v>
@@ -4969,31 +4969,31 @@
         <v>-1</v>
       </c>
       <c r="N85" s="2" t="n">
-        <v>-0.624951494613327</v>
+        <v>-0.3031502392603908</v>
       </c>
       <c r="O85" s="2" t="inlineStr">
         <is>
-          <t>above_ema60, ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, stronger_than_market, above_ichimoku_cloud</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" s="2" t="n">
-        <v>6464</v>
+        <v>6412</v>
       </c>
       <c r="B86" s="2" t="inlineStr">
         <is>
-          <t>台數科</t>
+          <t>群電</t>
         </is>
       </c>
       <c r="C86" s="2" t="n">
         <v/>
       </c>
       <c r="D86" s="2" t="n">
-        <v>416.0361574934307</v>
+        <v>423.3048338069732</v>
       </c>
       <c r="E86" s="2" t="n">
-        <v>77.7</v>
+        <v>93.09999999999999</v>
       </c>
       <c r="F86" s="2" t="inlineStr">
         <is>
@@ -5004,13 +5004,13 @@
         <v>0</v>
       </c>
       <c r="H86" s="2" t="n">
-        <v>47.48750627840681</v>
+        <v>49.05189400226433</v>
       </c>
       <c r="I86" s="2" t="n">
-        <v>14.49206111592081</v>
+        <v>19.53005845025127</v>
       </c>
       <c r="J86" s="2" t="n">
-        <v>0.0165331337309507</v>
+        <v>0.5443375335334363</v>
       </c>
       <c r="K86" s="2" t="n">
         <v>0</v>
@@ -5022,31 +5022,31 @@
         <v>-1</v>
       </c>
       <c r="N86" s="2" t="n">
-        <v>-0.0774135029241496</v>
+        <v>-0.624951494613327</v>
       </c>
       <c r="O86" s="2" t="inlineStr">
         <is>
-          <t>above_ema60, ema60_gt_ema120, market_above_ma60, avoid_chase, mfi_strong, above_ichimoku_cloud</t>
+          <t>above_ema60, ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, stronger_than_market, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" s="2" t="n">
-        <v>6225</v>
+        <v>6464</v>
       </c>
       <c r="B87" s="2" t="inlineStr">
         <is>
-          <t>天瀚</t>
+          <t>台數科</t>
         </is>
       </c>
       <c r="C87" s="2" t="n">
         <v/>
       </c>
       <c r="D87" s="2" t="n">
-        <v>394.1002912973766</v>
+        <v>416.0361574934307</v>
       </c>
       <c r="E87" s="2" t="n">
-        <v>20.35</v>
+        <v>77.7</v>
       </c>
       <c r="F87" s="2" t="inlineStr">
         <is>
@@ -5057,13 +5057,13 @@
         <v>0</v>
       </c>
       <c r="H87" s="2" t="n">
-        <v>36.16062328526709</v>
+        <v>47.48750627840681</v>
       </c>
       <c r="I87" s="2" t="n">
-        <v>12.24983934420584</v>
+        <v>14.49206111592081</v>
       </c>
       <c r="J87" s="2" t="n">
-        <v>3.175522031875905</v>
+        <v>0.0165331337309507</v>
       </c>
       <c r="K87" s="2" t="n">
         <v>0</v>
@@ -5075,31 +5075,31 @@
         <v>-1</v>
       </c>
       <c r="N87" s="2" t="n">
-        <v>-0.3594586943067883</v>
+        <v>-0.0774135029241496</v>
       </c>
       <c r="O87" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, volume_break, market_above_ma60, avoid_chase, mfi_strong</t>
+          <t>above_ema60, ema60_gt_ema120, market_above_ma60, avoid_chase, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" s="2" t="n">
-        <v>6170</v>
+        <v>6225</v>
       </c>
       <c r="B88" s="2" t="inlineStr">
         <is>
-          <t>統振</t>
+          <t>天瀚</t>
         </is>
       </c>
       <c r="C88" s="2" t="n">
         <v/>
       </c>
       <c r="D88" s="2" t="n">
-        <v>385.7444484967478</v>
+        <v>394.1002912973766</v>
       </c>
       <c r="E88" s="2" t="n">
-        <v>51.8</v>
+        <v>20.35</v>
       </c>
       <c r="F88" s="2" t="inlineStr">
         <is>
@@ -5110,13 +5110,13 @@
         <v>0</v>
       </c>
       <c r="H88" s="2" t="n">
-        <v>49.13738549243163</v>
+        <v>36.16062328526709</v>
       </c>
       <c r="I88" s="2" t="n">
-        <v>14.77398473219187</v>
+        <v>12.24983934420584</v>
       </c>
       <c r="J88" s="2" t="n">
-        <v>0.9561628634744944</v>
+        <v>3.175522031875905</v>
       </c>
       <c r="K88" s="2" t="n">
         <v>0</v>
@@ -5128,31 +5128,31 @@
         <v>-1</v>
       </c>
       <c r="N88" s="2" t="n">
-        <v>-0.0493571456995236</v>
+        <v>-0.3594586943067883</v>
       </c>
       <c r="O88" s="2" t="inlineStr">
         <is>
-          <t>above_ema60, ema60_gt_ema120, market_above_ma60, avoid_chase, mfi_strong, above_ichimoku_cloud</t>
+          <t>ema60_gt_ema120, volume_break, market_above_ma60, avoid_chase, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" s="2" t="n">
-        <v>6485</v>
+        <v>6170</v>
       </c>
       <c r="B89" s="2" t="inlineStr">
         <is>
-          <t>點序</t>
+          <t>統振</t>
         </is>
       </c>
       <c r="C89" s="2" t="n">
         <v/>
       </c>
       <c r="D89" s="2" t="n">
-        <v>382.7565161734089</v>
+        <v>385.7444484967478</v>
       </c>
       <c r="E89" s="2" t="n">
-        <v>88.09999999999999</v>
+        <v>51.8</v>
       </c>
       <c r="F89" s="2" t="inlineStr">
         <is>
@@ -5163,16 +5163,16 @@
         <v>0</v>
       </c>
       <c r="H89" s="2" t="n">
-        <v>42.9941961056934</v>
+        <v>49.13738549243163</v>
       </c>
       <c r="I89" s="2" t="n">
-        <v>18.50070578527776</v>
+        <v>14.77398473219187</v>
       </c>
       <c r="J89" s="2" t="n">
-        <v>0.2687442425150673</v>
+        <v>0.9561628634744944</v>
       </c>
       <c r="K89" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L89" s="2" t="n">
         <v>0</v>
@@ -5181,31 +5181,31 @@
         <v>-1</v>
       </c>
       <c r="N89" s="2" t="n">
-        <v>-1.793999783291008</v>
+        <v>-0.0493571456995236</v>
       </c>
       <c r="O89" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, kd_golden_cross, obv_uptrend</t>
+          <t>above_ema60, ema60_gt_ema120, market_above_ma60, avoid_chase, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" s="2" t="n">
-        <v>6426</v>
+        <v>6485</v>
       </c>
       <c r="B90" s="2" t="inlineStr">
         <is>
-          <t>統新</t>
+          <t>點序</t>
         </is>
       </c>
       <c r="C90" s="2" t="n">
         <v/>
       </c>
       <c r="D90" s="2" t="n">
-        <v>373.3266947893004</v>
+        <v>382.7565161734089</v>
       </c>
       <c r="E90" s="2" t="n">
-        <v>211.5</v>
+        <v>88.09999999999999</v>
       </c>
       <c r="F90" s="2" t="inlineStr">
         <is>
@@ -5216,13 +5216,13 @@
         <v>0</v>
       </c>
       <c r="H90" s="2" t="n">
-        <v>44.70606282070857</v>
+        <v>42.9941961056934</v>
       </c>
       <c r="I90" s="2" t="n">
-        <v>18.24177388833325</v>
+        <v>18.50070578527776</v>
       </c>
       <c r="J90" s="2" t="n">
-        <v>0.4107426598943384</v>
+        <v>0.2687442425150673</v>
       </c>
       <c r="K90" s="2" t="n">
         <v>1</v>
@@ -5234,31 +5234,31 @@
         <v>-1</v>
       </c>
       <c r="N90" s="2" t="n">
-        <v>-1.308762716848083</v>
+        <v>-1.793999783291008</v>
       </c>
       <c r="O90" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, liquidity_ok, stronger_than_market</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, kd_golden_cross, obv_uptrend</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" s="2" t="n">
-        <v>6165</v>
+        <v>6426</v>
       </c>
       <c r="B91" s="2" t="inlineStr">
         <is>
-          <t>浪凡</t>
+          <t>統新</t>
         </is>
       </c>
       <c r="C91" s="2" t="n">
         <v/>
       </c>
       <c r="D91" s="2" t="n">
-        <v>367.8868808010956</v>
+        <v>373.3266947893004</v>
       </c>
       <c r="E91" s="2" t="n">
-        <v>47.25</v>
+        <v>211.5</v>
       </c>
       <c r="F91" s="2" t="inlineStr">
         <is>
@@ -5269,16 +5269,16 @@
         <v>0</v>
       </c>
       <c r="H91" s="2" t="n">
-        <v>41.72454549391296</v>
+        <v>44.70606282070857</v>
       </c>
       <c r="I91" s="2" t="n">
-        <v>16.6635027513628</v>
+        <v>18.24177388833325</v>
       </c>
       <c r="J91" s="2" t="n">
-        <v>0.4026041610015554</v>
+        <v>0.4107426598943384</v>
       </c>
       <c r="K91" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L91" s="2" t="n">
         <v>0</v>
@@ -5287,31 +5287,31 @@
         <v>-1</v>
       </c>
       <c r="N91" s="2" t="n">
-        <v>-0.1795831456839571</v>
+        <v>-1.308762716848083</v>
       </c>
       <c r="O91" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, kd_golden_cross, mfi_strong</t>
+          <t>ema60_gt_ema120, market_above_ma60, liquidity_ok, stronger_than_market</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" s="2" t="n">
-        <v>6245</v>
+        <v>6165</v>
       </c>
       <c r="B92" s="2" t="inlineStr">
         <is>
-          <t>立端</t>
+          <t>浪凡</t>
         </is>
       </c>
       <c r="C92" s="2" t="n">
         <v/>
       </c>
       <c r="D92" s="2" t="n">
-        <v>352.2437294280718</v>
+        <v>367.8868808010956</v>
       </c>
       <c r="E92" s="2" t="n">
-        <v>80.40000000000001</v>
+        <v>47.25</v>
       </c>
       <c r="F92" s="2" t="inlineStr">
         <is>
@@ -5322,13 +5322,13 @@
         <v>0</v>
       </c>
       <c r="H92" s="2" t="n">
-        <v>41.52270874022156</v>
+        <v>41.72454549391296</v>
       </c>
       <c r="I92" s="2" t="n">
-        <v>17.38608337855748</v>
+        <v>16.6635027513628</v>
       </c>
       <c r="J92" s="2" t="n">
-        <v>0.4398700972799304</v>
+        <v>0.4026041610015554</v>
       </c>
       <c r="K92" s="2" t="n">
         <v>0</v>
@@ -5340,31 +5340,31 @@
         <v>-1</v>
       </c>
       <c r="N92" s="2" t="n">
-        <v>-0.7872150851782105</v>
+        <v>-0.1795831456839571</v>
       </c>
       <c r="O92" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, kd_golden_cross</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, kd_golden_cross, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" s="2" t="n">
-        <v>6205</v>
+        <v>6245</v>
       </c>
       <c r="B93" s="2" t="inlineStr">
         <is>
-          <t>詮欣</t>
+          <t>立端</t>
         </is>
       </c>
       <c r="C93" s="2" t="n">
         <v/>
       </c>
       <c r="D93" s="2" t="n">
-        <v>350.6823356060266</v>
+        <v>352.2437294280718</v>
       </c>
       <c r="E93" s="2" t="n">
-        <v>80.7</v>
+        <v>80.40000000000001</v>
       </c>
       <c r="F93" s="2" t="inlineStr">
         <is>
@@ -5375,13 +5375,13 @@
         <v>0</v>
       </c>
       <c r="H93" s="2" t="n">
-        <v>49.10599931280976</v>
+        <v>41.52270874022156</v>
       </c>
       <c r="I93" s="2" t="n">
-        <v>12.7701786745263</v>
+        <v>17.38608337855748</v>
       </c>
       <c r="J93" s="2" t="n">
-        <v>0.4364821385090437</v>
+        <v>0.4398700972799304</v>
       </c>
       <c r="K93" s="2" t="n">
         <v>0</v>
@@ -5393,31 +5393,31 @@
         <v>-1</v>
       </c>
       <c r="N93" s="2" t="n">
-        <v>-0.317414863854944</v>
+        <v>-0.7872150851782105</v>
       </c>
       <c r="O93" s="2" t="inlineStr">
         <is>
-          <t>above_ema60, ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, obv_uptrend</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, kd_golden_cross</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" s="2" t="n">
-        <v>6184</v>
+        <v>6205</v>
       </c>
       <c r="B94" s="2" t="inlineStr">
         <is>
-          <t>大豐電</t>
+          <t>詮欣</t>
         </is>
       </c>
       <c r="C94" s="2" t="n">
         <v/>
       </c>
       <c r="D94" s="2" t="n">
-        <v>350.575874683539</v>
+        <v>350.6823356060266</v>
       </c>
       <c r="E94" s="2" t="n">
-        <v>44.45</v>
+        <v>80.7</v>
       </c>
       <c r="F94" s="2" t="inlineStr">
         <is>
@@ -5428,16 +5428,16 @@
         <v>0</v>
       </c>
       <c r="H94" s="2" t="n">
-        <v>26.45721524033972</v>
+        <v>49.10599931280976</v>
       </c>
       <c r="I94" s="2" t="n">
-        <v>30.52637629833593</v>
+        <v>12.7701786745263</v>
       </c>
       <c r="J94" s="2" t="n">
-        <v>4.107410092097087</v>
+        <v>0.4364821385090437</v>
       </c>
       <c r="K94" s="2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="L94" s="2" t="n">
         <v>0</v>
@@ -5446,31 +5446,31 @@
         <v>-1</v>
       </c>
       <c r="N94" s="2" t="n">
-        <v>-0.0910398130198961</v>
+        <v>-0.317414863854944</v>
       </c>
       <c r="O94" s="2" t="inlineStr">
         <is>
-          <t>volume_break, market_above_ma60, avoid_chase, adx_trending</t>
+          <t>above_ema60, ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, obv_uptrend</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" s="2" t="n">
-        <v>6474</v>
+        <v>6184</v>
       </c>
       <c r="B95" s="2" t="inlineStr">
         <is>
-          <t>華豫寧</t>
+          <t>大豐電</t>
         </is>
       </c>
       <c r="C95" s="2" t="n">
         <v/>
       </c>
       <c r="D95" s="2" t="n">
-        <v>347.9365841319417</v>
+        <v>350.575874683539</v>
       </c>
       <c r="E95" s="2" t="n">
-        <v>37.7</v>
+        <v>44.45</v>
       </c>
       <c r="F95" s="2" t="inlineStr">
         <is>
@@ -5481,16 +5481,16 @@
         <v>0</v>
       </c>
       <c r="H95" s="2" t="n">
-        <v>51.49664881539967</v>
+        <v>26.45721524033972</v>
       </c>
       <c r="I95" s="2" t="n">
-        <v>17.23431749176274</v>
+        <v>30.52637629833593</v>
       </c>
       <c r="J95" s="2" t="n">
-        <v>0.6629715838702348</v>
+        <v>4.107410092097087</v>
       </c>
       <c r="K95" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L95" s="2" t="n">
         <v>0</v>
@@ -5499,31 +5499,31 @@
         <v>-1</v>
       </c>
       <c r="N95" s="2" t="n">
-        <v>0.4737497496088998</v>
+        <v>-0.0910398130198961</v>
       </c>
       <c r="O95" s="2" t="inlineStr">
         <is>
-          <t>above_ema60, market_above_ma60, avoid_chase, obv_uptrend, mfi_strong</t>
+          <t>volume_break, market_above_ma60, avoid_chase, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" s="2" t="n">
-        <v>6441</v>
+        <v>6474</v>
       </c>
       <c r="B96" s="2" t="inlineStr">
         <is>
-          <t>廣錠</t>
+          <t>華豫寧</t>
         </is>
       </c>
       <c r="C96" s="2" t="n">
         <v/>
       </c>
       <c r="D96" s="2" t="n">
-        <v>334.764272790886</v>
+        <v>347.9365841319417</v>
       </c>
       <c r="E96" s="2" t="n">
-        <v>22.2</v>
+        <v>37.7</v>
       </c>
       <c r="F96" s="2" t="inlineStr">
         <is>
@@ -5534,16 +5534,16 @@
         <v>0</v>
       </c>
       <c r="H96" s="2" t="n">
-        <v>42.03151405509114</v>
+        <v>51.49664881539967</v>
       </c>
       <c r="I96" s="2" t="n">
-        <v>10.5576951941934</v>
+        <v>17.23431749176274</v>
       </c>
       <c r="J96" s="2" t="n">
-        <v>0.452319178257975</v>
+        <v>0.6629715838702348</v>
       </c>
       <c r="K96" s="2" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="L96" s="2" t="n">
         <v>0</v>
@@ -5552,31 +5552,31 @@
         <v>-1</v>
       </c>
       <c r="N96" s="2" t="n">
-        <v>-0.1275098656446578</v>
+        <v>0.4737497496088998</v>
       </c>
       <c r="O96" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, foreign_buy_3d, mfi_strong</t>
+          <t>above_ema60, market_above_ma60, avoid_chase, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" s="2" t="n">
-        <v>6215</v>
+        <v>6441</v>
       </c>
       <c r="B97" s="2" t="inlineStr">
         <is>
-          <t>和椿</t>
+          <t>廣錠</t>
         </is>
       </c>
       <c r="C97" s="2" t="n">
         <v/>
       </c>
       <c r="D97" s="2" t="n">
-        <v>332.6789158752713</v>
+        <v>334.764272790886</v>
       </c>
       <c r="E97" s="2" t="n">
-        <v>106.5</v>
+        <v>22.2</v>
       </c>
       <c r="F97" s="2" t="inlineStr">
         <is>
@@ -5587,16 +5587,16 @@
         <v>0</v>
       </c>
       <c r="H97" s="2" t="n">
-        <v>40.56861180517854</v>
+        <v>42.03151405509114</v>
       </c>
       <c r="I97" s="2" t="n">
-        <v>19.57234940725234</v>
+        <v>10.5576951941934</v>
       </c>
       <c r="J97" s="2" t="n">
-        <v>0.3935708352004117</v>
+        <v>0.452319178257975</v>
       </c>
       <c r="K97" s="2" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="L97" s="2" t="n">
         <v>0</v>
@@ -5605,31 +5605,31 @@
         <v>-1</v>
       </c>
       <c r="N97" s="2" t="n">
-        <v>-0.9956584135950072</v>
+        <v>-0.1275098656446578</v>
       </c>
       <c r="O97" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, kd_golden_cross</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, foreign_buy_3d, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" s="2" t="n">
-        <v>6201</v>
+        <v>6215</v>
       </c>
       <c r="B98" s="2" t="inlineStr">
         <is>
-          <t>亞弘電</t>
+          <t>和椿</t>
         </is>
       </c>
       <c r="C98" s="2" t="n">
         <v/>
       </c>
       <c r="D98" s="2" t="n">
-        <v>274.4068679807692</v>
+        <v>332.6789158752713</v>
       </c>
       <c r="E98" s="2" t="n">
-        <v>48.65</v>
+        <v>106.5</v>
       </c>
       <c r="F98" s="2" t="inlineStr">
         <is>
@@ -5640,16 +5640,16 @@
         <v>0</v>
       </c>
       <c r="H98" s="2" t="n">
-        <v>52.803646670909</v>
+        <v>40.56861180517854</v>
       </c>
       <c r="I98" s="2" t="n">
-        <v>15.8117676754197</v>
+        <v>19.57234940725234</v>
       </c>
       <c r="J98" s="2" t="n">
-        <v>0.027158009005024</v>
+        <v>0.3935708352004117</v>
       </c>
       <c r="K98" s="2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="L98" s="2" t="n">
         <v>0</v>
@@ -5658,31 +5658,31 @@
         <v>-1</v>
       </c>
       <c r="N98" s="2" t="n">
-        <v>0.1777125808474383</v>
+        <v>-0.9956584135950072</v>
       </c>
       <c r="O98" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, stronger_than_market, mfi_strong</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, kd_golden_cross</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" s="2" t="n">
-        <v>6416</v>
+        <v>6201</v>
       </c>
       <c r="B99" s="2" t="inlineStr">
         <is>
-          <t>瑞祺電通</t>
+          <t>亞弘電</t>
         </is>
       </c>
       <c r="C99" s="2" t="n">
         <v/>
       </c>
       <c r="D99" s="2" t="n">
-        <v>266.0720666084964</v>
+        <v>274.4068679807692</v>
       </c>
       <c r="E99" s="2" t="n">
-        <v>82</v>
+        <v>48.65</v>
       </c>
       <c r="F99" s="2" t="inlineStr">
         <is>
@@ -5693,16 +5693,16 @@
         <v>0</v>
       </c>
       <c r="H99" s="2" t="n">
-        <v>40.45936833036081</v>
+        <v>52.803646670909</v>
       </c>
       <c r="I99" s="2" t="n">
-        <v>22.26309679639846</v>
+        <v>15.8117676754197</v>
       </c>
       <c r="J99" s="2" t="n">
-        <v>0.6738776381873547</v>
+        <v>0.027158009005024</v>
       </c>
       <c r="K99" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L99" s="2" t="n">
         <v>0</v>
@@ -5711,31 +5711,31 @@
         <v>-1</v>
       </c>
       <c r="N99" s="2" t="n">
-        <v>-0.5157206705231719</v>
+        <v>0.1777125808474383</v>
       </c>
       <c r="O99" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, adx_trending</t>
+          <t>market_above_ma60, avoid_chase, stronger_than_market, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" s="2" t="n">
-        <v>6266</v>
+        <v>6416</v>
       </c>
       <c r="B100" s="2" t="inlineStr">
         <is>
-          <t>泰詠</t>
+          <t>瑞祺電通</t>
         </is>
       </c>
       <c r="C100" s="2" t="n">
         <v/>
       </c>
       <c r="D100" s="2" t="n">
-        <v>256.5116330556198</v>
+        <v>266.0720666084964</v>
       </c>
       <c r="E100" s="2" t="n">
-        <v>25.55</v>
+        <v>82</v>
       </c>
       <c r="F100" s="2" t="inlineStr">
         <is>
@@ -5746,16 +5746,16 @@
         <v>0</v>
       </c>
       <c r="H100" s="2" t="n">
-        <v>35.65646524089885</v>
+        <v>40.45936833036081</v>
       </c>
       <c r="I100" s="2" t="n">
-        <v>23.00289922637265</v>
+        <v>22.26309679639846</v>
       </c>
       <c r="J100" s="2" t="n">
-        <v>0.393402586773683</v>
+        <v>0.6738776381873547</v>
       </c>
       <c r="K100" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L100" s="2" t="n">
         <v>0</v>
@@ -5764,31 +5764,31 @@
         <v>-1</v>
       </c>
       <c r="N100" s="2" t="n">
-        <v>-0.1264377484889248</v>
+        <v>-0.5157206705231719</v>
       </c>
       <c r="O100" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, adx_trending, kd_golden_cross</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" s="2" t="n">
-        <v>6276</v>
+        <v>6266</v>
       </c>
       <c r="B101" s="2" t="inlineStr">
         <is>
-          <t>安鈦克</t>
+          <t>泰詠</t>
         </is>
       </c>
       <c r="C101" s="2" t="n">
         <v/>
       </c>
       <c r="D101" s="2" t="n">
-        <v>254.9235034826114</v>
+        <v>256.5116330556198</v>
       </c>
       <c r="E101" s="2" t="n">
-        <v>22.55</v>
+        <v>25.55</v>
       </c>
       <c r="F101" s="2" t="inlineStr">
         <is>
@@ -5799,13 +5799,13 @@
         <v>0</v>
       </c>
       <c r="H101" s="2" t="n">
-        <v>26.74590521459301</v>
+        <v>35.65646524089885</v>
       </c>
       <c r="I101" s="2" t="n">
-        <v>24.86651591713715</v>
+        <v>23.00289922637265</v>
       </c>
       <c r="J101" s="2" t="n">
-        <v>2.871033009854247</v>
+        <v>0.393402586773683</v>
       </c>
       <c r="K101" s="2" t="n">
         <v>0</v>
@@ -5817,31 +5817,31 @@
         <v>-1</v>
       </c>
       <c r="N101" s="2" t="n">
-        <v>-0.209926166769665</v>
+        <v>-0.1264377484889248</v>
       </c>
       <c r="O101" s="2" t="inlineStr">
         <is>
-          <t>volume_break, market_above_ma60, avoid_chase, adx_trending</t>
+          <t>market_above_ma60, avoid_chase, adx_trending, kd_golden_cross</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" s="2" t="n">
-        <v>6210</v>
+        <v>6276</v>
       </c>
       <c r="B102" s="2" t="inlineStr">
         <is>
-          <t>慶生</t>
+          <t>安鈦克</t>
         </is>
       </c>
       <c r="C102" s="2" t="n">
         <v/>
       </c>
       <c r="D102" s="2" t="n">
-        <v>235.2812910420709</v>
+        <v>254.9235034826113</v>
       </c>
       <c r="E102" s="2" t="n">
-        <v>20.5</v>
+        <v>22.55</v>
       </c>
       <c r="F102" s="2" t="inlineStr">
         <is>
@@ -5852,13 +5852,13 @@
         <v>0</v>
       </c>
       <c r="H102" s="2" t="n">
-        <v>45.41332627091635</v>
+        <v>26.74590521459301</v>
       </c>
       <c r="I102" s="2" t="n">
-        <v>17.92137974585088</v>
+        <v>24.86651591713715</v>
       </c>
       <c r="J102" s="2" t="n">
-        <v>0.3539206443055977</v>
+        <v>2.871033009854247</v>
       </c>
       <c r="K102" s="2" t="n">
         <v>0</v>
@@ -5870,31 +5870,31 @@
         <v>-1</v>
       </c>
       <c r="N102" s="2" t="n">
-        <v>-0.0815970251819756</v>
+        <v>-0.209926166769665</v>
       </c>
       <c r="O102" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase</t>
+          <t>volume_break, market_above_ma60, avoid_chase, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" s="2" t="n">
-        <v>6191</v>
+        <v>6210</v>
       </c>
       <c r="B103" s="2" t="inlineStr">
         <is>
-          <t>精成科</t>
+          <t>慶生</t>
         </is>
       </c>
       <c r="C103" s="2" t="n">
         <v/>
       </c>
       <c r="D103" s="2" t="n">
-        <v>224.5500235497685</v>
+        <v>235.2812910420709</v>
       </c>
       <c r="E103" s="2" t="n">
-        <v>98.40000000000001</v>
+        <v>20.5</v>
       </c>
       <c r="F103" s="2" t="inlineStr">
         <is>
@@ -5905,13 +5905,13 @@
         <v>0</v>
       </c>
       <c r="H103" s="2" t="n">
-        <v>50.32460456069935</v>
+        <v>45.41332627091635</v>
       </c>
       <c r="I103" s="2" t="n">
-        <v>17.52318665884046</v>
+        <v>17.92137974585088</v>
       </c>
       <c r="J103" s="2" t="n">
-        <v>0.5065204386442225</v>
+        <v>0.3539206443055977</v>
       </c>
       <c r="K103" s="2" t="n">
         <v>0</v>
@@ -5923,31 +5923,31 @@
         <v>-1</v>
       </c>
       <c r="N103" s="2" t="n">
-        <v>0.3905905252100806</v>
+        <v>-0.0815970251819756</v>
       </c>
       <c r="O103" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, liquidity_ok, mfi_strong</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" s="2" t="n">
-        <v>6203</v>
+        <v>6191</v>
       </c>
       <c r="B104" s="2" t="inlineStr">
         <is>
-          <t>海韻電</t>
+          <t>精成科</t>
         </is>
       </c>
       <c r="C104" s="2" t="n">
         <v/>
       </c>
       <c r="D104" s="2" t="n">
-        <v>224.2907066001358</v>
+        <v>224.5500235497685</v>
       </c>
       <c r="E104" s="2" t="n">
-        <v>67.3</v>
+        <v>98.40000000000001</v>
       </c>
       <c r="F104" s="2" t="inlineStr">
         <is>
@@ -5958,13 +5958,13 @@
         <v>0</v>
       </c>
       <c r="H104" s="2" t="n">
-        <v>43.16970137394868</v>
+        <v>50.32460456069935</v>
       </c>
       <c r="I104" s="2" t="n">
-        <v>20.24075769892589</v>
+        <v>17.52318665884046</v>
       </c>
       <c r="J104" s="2" t="n">
-        <v>0.7694609042831414</v>
+        <v>0.5065204386442225</v>
       </c>
       <c r="K104" s="2" t="n">
         <v>0</v>
@@ -5976,31 +5976,31 @@
         <v>-1</v>
       </c>
       <c r="N104" s="2" t="n">
-        <v>-0.2532659191781334</v>
+        <v>0.3905905252100806</v>
       </c>
       <c r="O104" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, adx_trending</t>
+          <t>market_above_ma60, avoid_chase, liquidity_ok, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" s="2" t="n">
-        <v>6443</v>
+        <v>6203</v>
       </c>
       <c r="B105" s="2" t="inlineStr">
         <is>
-          <t>元晶</t>
+          <t>海韻電</t>
         </is>
       </c>
       <c r="C105" s="2" t="n">
         <v/>
       </c>
       <c r="D105" s="2" t="n">
-        <v>210.4212422207024</v>
+        <v>224.2907066001358</v>
       </c>
       <c r="E105" s="2" t="n">
-        <v>37.05</v>
+        <v>67.3</v>
       </c>
       <c r="F105" s="2" t="inlineStr">
         <is>
@@ -6011,13 +6011,13 @@
         <v>0</v>
       </c>
       <c r="H105" s="2" t="n">
-        <v>41.23955540639028</v>
+        <v>43.16970137394868</v>
       </c>
       <c r="I105" s="2" t="n">
-        <v>16.62226347040148</v>
+        <v>20.24075769892589</v>
       </c>
       <c r="J105" s="2" t="n">
-        <v>0.3228717873546574</v>
+        <v>0.7694609042831414</v>
       </c>
       <c r="K105" s="2" t="n">
         <v>0</v>
@@ -6029,31 +6029,31 @@
         <v>-1</v>
       </c>
       <c r="N105" s="2" t="n">
-        <v>-0.3836254858037361</v>
+        <v>-0.2532659191781334</v>
       </c>
       <c r="O105" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="106">
       <c r="A106" s="2" t="n">
-        <v>6230</v>
+        <v>6443</v>
       </c>
       <c r="B106" s="2" t="inlineStr">
         <is>
-          <t>尼得科超眾</t>
+          <t>元晶</t>
         </is>
       </c>
       <c r="C106" s="2" t="n">
         <v/>
       </c>
       <c r="D106" s="2" t="n">
-        <v>201.8482366886569</v>
+        <v>210.4212422207024</v>
       </c>
       <c r="E106" s="2" t="n">
-        <v>131</v>
+        <v>37.05</v>
       </c>
       <c r="F106" s="2" t="inlineStr">
         <is>
@@ -6064,13 +6064,13 @@
         <v>0</v>
       </c>
       <c r="H106" s="2" t="n">
-        <v>41.38718910956901</v>
+        <v>41.23955540639028</v>
       </c>
       <c r="I106" s="2" t="n">
-        <v>11.19032130628412</v>
+        <v>16.62226347040148</v>
       </c>
       <c r="J106" s="2" t="n">
-        <v>0.4492893674320194</v>
+        <v>0.3228717873546574</v>
       </c>
       <c r="K106" s="2" t="n">
         <v>0</v>
@@ -6082,48 +6082,48 @@
         <v>-1</v>
       </c>
       <c r="N106" s="2" t="n">
-        <v>0.1247034041355856</v>
+        <v>-0.3836254858037361</v>
       </c>
       <c r="O106" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok</t>
         </is>
       </c>
     </row>
     <row r="107">
       <c r="A107" s="2" t="n">
-        <v>6287</v>
+        <v>6230</v>
       </c>
       <c r="B107" s="2" t="inlineStr">
         <is>
-          <t>元隆</t>
+          <t>尼得科超眾</t>
         </is>
       </c>
       <c r="C107" s="2" t="n">
         <v/>
       </c>
       <c r="D107" s="2" t="n">
-        <v>201.4669994133625</v>
+        <v>201.8482366886569</v>
       </c>
       <c r="E107" s="2" t="n">
-        <v>8.890000000000001</v>
+        <v>131</v>
       </c>
       <c r="F107" s="2" t="inlineStr">
         <is>
-          <t>2025-06-20</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="G107" s="2" t="b">
         <v>0</v>
       </c>
       <c r="H107" s="2" t="n">
-        <v>51.71399387501272</v>
+        <v>41.38718910956901</v>
       </c>
       <c r="I107" s="2" t="n">
-        <v>0.9229390487499936</v>
+        <v>11.19032130628412</v>
       </c>
       <c r="J107" s="2" t="n">
-        <v>0.3819364013941486</v>
+        <v>0.4492893674320194</v>
       </c>
       <c r="K107" s="2" t="n">
         <v>0</v>
@@ -6135,51 +6135,51 @@
         <v>-1</v>
       </c>
       <c r="N107" s="2" t="n">
-        <v>-0.0153085825903483</v>
+        <v>0.1247034041355856</v>
       </c>
       <c r="O107" s="2" t="inlineStr">
         <is>
-          <t>above_ema60, avoid_chase, obv_uptrend</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase</t>
         </is>
       </c>
     </row>
     <row r="108">
       <c r="A108" s="2" t="n">
-        <v>6188</v>
+        <v>6287</v>
       </c>
       <c r="B108" s="2" t="inlineStr">
         <is>
-          <t>廣明</t>
+          <t>元隆</t>
         </is>
       </c>
       <c r="C108" s="2" t="n">
         <v/>
       </c>
       <c r="D108" s="2" t="n">
-        <v>195.152856634918</v>
+        <v>201.4669994133625</v>
       </c>
       <c r="E108" s="2" t="n">
-        <v>78.5</v>
+        <v>8.890000000000001</v>
       </c>
       <c r="F108" s="2" t="inlineStr">
         <is>
-          <t>2026-06-24</t>
+          <t>2025-06-20</t>
         </is>
       </c>
       <c r="G108" s="2" t="b">
         <v>0</v>
       </c>
       <c r="H108" s="2" t="n">
-        <v>41.1874483270002</v>
+        <v>51.71399387501272</v>
       </c>
       <c r="I108" s="2" t="n">
-        <v>14.3143088524894</v>
+        <v>0.9229390487499936</v>
       </c>
       <c r="J108" s="2" t="n">
-        <v>0.458902430936417</v>
+        <v>0.3819364013941486</v>
       </c>
       <c r="K108" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L108" s="2" t="n">
         <v>0</v>
@@ -6188,31 +6188,31 @@
         <v>-1</v>
       </c>
       <c r="N108" s="2" t="n">
-        <v>-0.2933120524136325</v>
+        <v>-0.0153085825903483</v>
       </c>
       <c r="O108" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, liquidity_ok, kd_golden_cross</t>
+          <t>above_ema60, avoid_chase, obv_uptrend</t>
         </is>
       </c>
     </row>
     <row r="109">
       <c r="A109" s="2" t="n">
-        <v>6272</v>
+        <v>6188</v>
       </c>
       <c r="B109" s="2" t="inlineStr">
         <is>
-          <t>驊陞</t>
+          <t>廣明</t>
         </is>
       </c>
       <c r="C109" s="2" t="n">
         <v/>
       </c>
       <c r="D109" s="2" t="n">
-        <v>189.6958974040213</v>
+        <v>195.152856634918</v>
       </c>
       <c r="E109" s="2" t="n">
-        <v>31.4</v>
+        <v>78.5</v>
       </c>
       <c r="F109" s="2" t="inlineStr">
         <is>
@@ -6223,16 +6223,16 @@
         <v>0</v>
       </c>
       <c r="H109" s="2" t="n">
-        <v>37.03153027939226</v>
+        <v>41.1874483270002</v>
       </c>
       <c r="I109" s="2" t="n">
-        <v>25.97219101528298</v>
+        <v>14.3143088524894</v>
       </c>
       <c r="J109" s="2" t="n">
-        <v>0.5665265176714727</v>
+        <v>0.458902430936417</v>
       </c>
       <c r="K109" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L109" s="2" t="n">
         <v>0</v>
@@ -6241,31 +6241,31 @@
         <v>-1</v>
       </c>
       <c r="N109" s="2" t="n">
-        <v>-0.6224787127616496</v>
+        <v>-0.2933120524136325</v>
       </c>
       <c r="O109" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, adx_trending</t>
+          <t>market_above_ma60, avoid_chase, liquidity_ok, kd_golden_cross</t>
         </is>
       </c>
     </row>
     <row r="110">
       <c r="A110" s="2" t="n">
-        <v>6281</v>
+        <v>6272</v>
       </c>
       <c r="B110" s="2" t="inlineStr">
         <is>
-          <t>全國電</t>
+          <t>驊陞</t>
         </is>
       </c>
       <c r="C110" s="2" t="n">
         <v/>
       </c>
       <c r="D110" s="2" t="n">
-        <v>180.4887721188194</v>
+        <v>189.6958974040213</v>
       </c>
       <c r="E110" s="2" t="n">
-        <v>51.2</v>
+        <v>31.4</v>
       </c>
       <c r="F110" s="2" t="inlineStr">
         <is>
@@ -6276,16 +6276,16 @@
         <v>0</v>
       </c>
       <c r="H110" s="2" t="n">
-        <v>47.80372122277673</v>
+        <v>37.03153027939226</v>
       </c>
       <c r="I110" s="2" t="n">
-        <v>12.15905165903494</v>
+        <v>25.97219101528298</v>
       </c>
       <c r="J110" s="2" t="n">
-        <v>0.6966117058334395</v>
+        <v>0.5665265176714727</v>
       </c>
       <c r="K110" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L110" s="2" t="n">
         <v>0</v>
@@ -6294,31 +6294,31 @@
         <v>-1</v>
       </c>
       <c r="N110" s="2" t="n">
-        <v>0.0257435635275203</v>
+        <v>-0.6224787127616496</v>
       </c>
       <c r="O110" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, mfi_strong</t>
+          <t>market_above_ma60, avoid_chase, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="111">
       <c r="A111" s="2" t="n">
-        <v>6477</v>
+        <v>6281</v>
       </c>
       <c r="B111" s="2" t="inlineStr">
         <is>
-          <t>安集</t>
+          <t>全國電</t>
         </is>
       </c>
       <c r="C111" s="2" t="n">
         <v/>
       </c>
       <c r="D111" s="2" t="n">
-        <v>169.6436016037619</v>
+        <v>180.4887721188194</v>
       </c>
       <c r="E111" s="2" t="n">
-        <v>31.8</v>
+        <v>51.2</v>
       </c>
       <c r="F111" s="2" t="inlineStr">
         <is>
@@ -6329,16 +6329,16 @@
         <v>0</v>
       </c>
       <c r="H111" s="2" t="n">
-        <v>42.40609583194681</v>
+        <v>47.80372122277673</v>
       </c>
       <c r="I111" s="2" t="n">
-        <v>13.04206146125356</v>
+        <v>12.15905165903494</v>
       </c>
       <c r="J111" s="2" t="n">
-        <v>0.3286537002825329</v>
+        <v>0.6966117058334395</v>
       </c>
       <c r="K111" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L111" s="2" t="n">
         <v>0</v>
@@ -6347,7 +6347,7 @@
         <v>-1</v>
       </c>
       <c r="N111" s="2" t="n">
-        <v>-0.134554575661616</v>
+        <v>0.0257435635275203</v>
       </c>
       <c r="O111" s="2" t="inlineStr">
         <is>
@@ -6357,21 +6357,21 @@
     </row>
     <row r="112">
       <c r="A112" s="2" t="n">
-        <v>6194</v>
+        <v>6477</v>
       </c>
       <c r="B112" s="2" t="inlineStr">
         <is>
-          <t>育富</t>
+          <t>安集</t>
         </is>
       </c>
       <c r="C112" s="2" t="n">
         <v/>
       </c>
       <c r="D112" s="2" t="n">
-        <v>163.6772189937627</v>
+        <v>169.6436016037619</v>
       </c>
       <c r="E112" s="2" t="n">
-        <v>32.3</v>
+        <v>31.8</v>
       </c>
       <c r="F112" s="2" t="inlineStr">
         <is>
@@ -6382,16 +6382,16 @@
         <v>0</v>
       </c>
       <c r="H112" s="2" t="n">
-        <v>43.39947501725723</v>
+        <v>42.40609583194681</v>
       </c>
       <c r="I112" s="2" t="n">
-        <v>16.14654180573206</v>
+        <v>13.04206146125356</v>
       </c>
       <c r="J112" s="2" t="n">
-        <v>0.4401263171258093</v>
+        <v>0.3286537002825329</v>
       </c>
       <c r="K112" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L112" s="2" t="n">
         <v>0</v>
@@ -6400,31 +6400,31 @@
         <v>-1</v>
       </c>
       <c r="N112" s="2" t="n">
-        <v>-0.1318138534737122</v>
+        <v>-0.134554575661616</v>
       </c>
       <c r="O112" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, kd_golden_cross</t>
+          <t>market_above_ma60, avoid_chase, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="113">
       <c r="A113" s="2" t="n">
-        <v>6183</v>
+        <v>6194</v>
       </c>
       <c r="B113" s="2" t="inlineStr">
         <is>
-          <t>關貿</t>
+          <t>育富</t>
         </is>
       </c>
       <c r="C113" s="2" t="n">
         <v/>
       </c>
       <c r="D113" s="2" t="n">
-        <v>156.4868503113821</v>
+        <v>163.6772189937627</v>
       </c>
       <c r="E113" s="2" t="n">
-        <v>90.3</v>
+        <v>32.3</v>
       </c>
       <c r="F113" s="2" t="inlineStr">
         <is>
@@ -6435,16 +6435,16 @@
         <v>0</v>
       </c>
       <c r="H113" s="2" t="n">
-        <v>47.39243440650005</v>
+        <v>43.39947501725723</v>
       </c>
       <c r="I113" s="2" t="n">
-        <v>14.61426480104285</v>
+        <v>16.14654180573206</v>
       </c>
       <c r="J113" s="2" t="n">
-        <v>0.3372991179078703</v>
+        <v>0.4401263171258093</v>
       </c>
       <c r="K113" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L113" s="2" t="n">
         <v>0</v>
@@ -6453,31 +6453,31 @@
         <v>-1</v>
       </c>
       <c r="N113" s="2" t="n">
-        <v>0.1550121678240335</v>
+        <v>-0.1318138534737122</v>
       </c>
       <c r="O113" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase</t>
+          <t>market_above_ma60, avoid_chase, kd_golden_cross</t>
         </is>
       </c>
     </row>
     <row r="114">
       <c r="A114" s="2" t="n">
-        <v>6235</v>
+        <v>6183</v>
       </c>
       <c r="B114" s="2" t="inlineStr">
         <is>
-          <t>華孚</t>
+          <t>關貿</t>
         </is>
       </c>
       <c r="C114" s="2" t="n">
         <v/>
       </c>
       <c r="D114" s="2" t="n">
-        <v>147.904271325607</v>
+        <v>156.4868503113821</v>
       </c>
       <c r="E114" s="2" t="n">
-        <v>40.5</v>
+        <v>90.3</v>
       </c>
       <c r="F114" s="2" t="inlineStr">
         <is>
@@ -6488,13 +6488,13 @@
         <v>0</v>
       </c>
       <c r="H114" s="2" t="n">
-        <v>43.10248366032674</v>
+        <v>47.39243440650005</v>
       </c>
       <c r="I114" s="2" t="n">
-        <v>14.21930433383427</v>
+        <v>14.61426480104285</v>
       </c>
       <c r="J114" s="2" t="n">
-        <v>0.3096077881547118</v>
+        <v>0.3372991179078703</v>
       </c>
       <c r="K114" s="2" t="n">
         <v>0</v>
@@ -6506,62 +6506,115 @@
         <v>-1</v>
       </c>
       <c r="N114" s="2" t="n">
-        <v>-0.1316735639391921</v>
+        <v>0.1550121678240335</v>
       </c>
       <c r="O114" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, liquidity_ok</t>
+          <t>market_above_ma60, avoid_chase</t>
         </is>
       </c>
     </row>
     <row r="115">
       <c r="A115" s="2" t="n">
+        <v>6235</v>
+      </c>
+      <c r="B115" s="2" t="inlineStr">
+        <is>
+          <t>華孚</t>
+        </is>
+      </c>
+      <c r="C115" s="2" t="n">
+        <v/>
+      </c>
+      <c r="D115" s="2" t="n">
+        <v>147.904271325607</v>
+      </c>
+      <c r="E115" s="2" t="n">
+        <v>40.5</v>
+      </c>
+      <c r="F115" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="G115" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="H115" s="2" t="n">
+        <v>43.10248366032674</v>
+      </c>
+      <c r="I115" s="2" t="n">
+        <v>14.21930433383427</v>
+      </c>
+      <c r="J115" s="2" t="n">
+        <v>0.3096077881547118</v>
+      </c>
+      <c r="K115" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L115" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M115" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="N115" s="2" t="n">
+        <v>-0.1316735639391921</v>
+      </c>
+      <c r="O115" s="2" t="inlineStr">
+        <is>
+          <t>market_above_ma60, avoid_chase, liquidity_ok</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" s="2" t="n">
         <v>6236</v>
       </c>
-      <c r="B115" s="2" t="inlineStr">
+      <c r="B116" s="2" t="inlineStr">
         <is>
           <t>中湛</t>
         </is>
       </c>
-      <c r="C115" s="2" t="n">
-        <v/>
-      </c>
-      <c r="D115" s="2" t="n">
+      <c r="C116" s="2" t="n">
+        <v/>
+      </c>
+      <c r="D116" s="2" t="n">
         <v>109.1137018383864</v>
       </c>
-      <c r="E115" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="F115" s="2" t="inlineStr">
-        <is>
-          <t>2026-06-24</t>
-        </is>
-      </c>
-      <c r="G115" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="H115" s="2" t="n">
+      <c r="E116" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F116" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="G116" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="H116" s="2" t="n">
         <v>48.0262578347586</v>
       </c>
-      <c r="I115" s="2" t="n">
+      <c r="I116" s="2" t="n">
         <v>7.290535660757568</v>
       </c>
-      <c r="J115" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="K115" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="L115" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="M115" s="2" t="n">
-        <v>-1</v>
-      </c>
-      <c r="N115" s="2" t="n">
+      <c r="J116" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K116" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L116" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M116" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="N116" s="2" t="n">
         <v>-0.346420649877792</v>
       </c>
-      <c r="O115" s="2" t="inlineStr">
+      <c r="O116" s="2" t="inlineStr">
         <is>
           <t>market_above_ma60, obv_uptrend</t>
         </is>

</xml_diff>